<commit_message>
fix: make member import codes client friendly
</commit_message>
<xml_diff>
--- a/public/templates/we-discipline-reprise-membres.xlsx
+++ b/public/templates/we-discipline-reprise-membres.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Membres" sheetId="1" r:id="Re6865aecd4db4dbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="2" r:id="Rd21582141b7b4ed0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" r:id="R2cf4116144174a3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Membres" sheetId="1" r:id="Rfa0de04aca884ea6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="2" r:id="Rfb1309f014064da1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" r:id="Ra72fa7b02cec4ead"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -281,7 +281,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
@@ -307,7 +307,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="2" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Code membre (auto)</x:v>
       </x:c>
       <x:c r="B1" s="2" t="str">
         <x:v>Prénom</x:v>
@@ -7359,6 +7359,9 @@
       <x:c r="S500" s="6"/>
       <x:c r="T500" s="4"/>
     </x:row>
+    <x:row r="501">
+      <x:c r="A501"/>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="D2:D500">

</xml_diff>

<commit_message>
fix: simplify bulk import auto member code
</commit_message>
<xml_diff>
--- a/public/templates/we-discipline-reprise-membres.xlsx
+++ b/public/templates/we-discipline-reprise-membres.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Membres" sheetId="1" r:id="Red17d53564064cb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exemple" sheetId="2" r:id="R96c66683005a4317"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="3" r:id="R4d51fb8564ff4ef3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aide" sheetId="4" r:id="R873bdf8d12c4487c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compatibilite" sheetId="5" r:id="R68b96b4b7fa145f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Membres" sheetId="1" r:id="R3860d04ca1d84e04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exemple" sheetId="2" r:id="Rd1071e9dbe554272"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="3" r:id="R67e59fb05a194423"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aide" sheetId="4" r:id="R55f36f945d164978"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compatibilite" sheetId="5" r:id="Rdf1066b99da04ff3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -451,7 +451,7 @@
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A1" s="12" t="str">
-        <x:v>Référence auto (optionnel)</x:v>
+        <x:v>Code membre auto</x:v>
       </x:c>
       <x:c r="B1" s="13" t="str">
         <x:v>Prénom</x:v>
@@ -519,7 +519,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="16" t="str">
-        <x:f>IF(AND(B2="",C2=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B2&amp;C2," ",""))&amp;IF(E2&lt;&gt;"","-"&amp;RIGHT(E2,4),IF(J2&lt;&gt;"","-"&amp;RIGHT(J2,4),"")))</x:f>
+        <x:f>IF(AND(B2="",C2=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B2&amp;C2," ",""))&amp;IF(E2&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E2," ",""),4),IF(J2&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J2," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B2" s="16"/>
       <x:c r="C2" s="16"/>
@@ -545,7 +545,7 @@
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="16" t="str">
-        <x:f>IF(AND(B3="",C3=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B3&amp;C3," ",""))&amp;IF(E3&lt;&gt;"","-"&amp;RIGHT(E3,4),IF(J3&lt;&gt;"","-"&amp;RIGHT(J3,4),"")))</x:f>
+        <x:f>IF(AND(B3="",C3=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B3&amp;C3," ",""))&amp;IF(E3&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E3," ",""),4),IF(J3&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J3," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B3" s="16"/>
       <x:c r="C3" s="16"/>
@@ -571,7 +571,7 @@
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="16" t="str">
-        <x:f>IF(AND(B4="",C4=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B4&amp;C4," ",""))&amp;IF(E4&lt;&gt;"","-"&amp;RIGHT(E4,4),IF(J4&lt;&gt;"","-"&amp;RIGHT(J4,4),"")))</x:f>
+        <x:f>IF(AND(B4="",C4=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B4&amp;C4," ",""))&amp;IF(E4&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E4," ",""),4),IF(J4&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J4," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B4" s="16"/>
       <x:c r="C4" s="16"/>
@@ -597,7 +597,7 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="16" t="str">
-        <x:f>IF(AND(B5="",C5=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B5&amp;C5," ",""))&amp;IF(E5&lt;&gt;"","-"&amp;RIGHT(E5,4),IF(J5&lt;&gt;"","-"&amp;RIGHT(J5,4),"")))</x:f>
+        <x:f>IF(AND(B5="",C5=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B5&amp;C5," ",""))&amp;IF(E5&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E5," ",""),4),IF(J5&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J5," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B5" s="16"/>
       <x:c r="C5" s="16"/>
@@ -623,7 +623,7 @@
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="16" t="str">
-        <x:f>IF(AND(B6="",C6=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B6&amp;C6," ",""))&amp;IF(E6&lt;&gt;"","-"&amp;RIGHT(E6,4),IF(J6&lt;&gt;"","-"&amp;RIGHT(J6,4),"")))</x:f>
+        <x:f>IF(AND(B6="",C6=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B6&amp;C6," ",""))&amp;IF(E6&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E6," ",""),4),IF(J6&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J6," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B6" s="16"/>
       <x:c r="C6" s="16"/>
@@ -649,7 +649,7 @@
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="16" t="str">
-        <x:f>IF(AND(B7="",C7=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B7&amp;C7," ",""))&amp;IF(E7&lt;&gt;"","-"&amp;RIGHT(E7,4),IF(J7&lt;&gt;"","-"&amp;RIGHT(J7,4),"")))</x:f>
+        <x:f>IF(AND(B7="",C7=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B7&amp;C7," ",""))&amp;IF(E7&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E7," ",""),4),IF(J7&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J7," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B7" s="16"/>
       <x:c r="C7" s="16"/>
@@ -675,7 +675,7 @@
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="16" t="str">
-        <x:f>IF(AND(B8="",C8=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B8&amp;C8," ",""))&amp;IF(E8&lt;&gt;"","-"&amp;RIGHT(E8,4),IF(J8&lt;&gt;"","-"&amp;RIGHT(J8,4),"")))</x:f>
+        <x:f>IF(AND(B8="",C8=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B8&amp;C8," ",""))&amp;IF(E8&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E8," ",""),4),IF(J8&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J8," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B8" s="16"/>
       <x:c r="C8" s="16"/>
@@ -701,7 +701,7 @@
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="16" t="str">
-        <x:f>IF(AND(B9="",C9=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B9&amp;C9," ",""))&amp;IF(E9&lt;&gt;"","-"&amp;RIGHT(E9,4),IF(J9&lt;&gt;"","-"&amp;RIGHT(J9,4),"")))</x:f>
+        <x:f>IF(AND(B9="",C9=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B9&amp;C9," ",""))&amp;IF(E9&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E9," ",""),4),IF(J9&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J9," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B9" s="16"/>
       <x:c r="C9" s="16"/>
@@ -727,7 +727,7 @@
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="16" t="str">
-        <x:f>IF(AND(B10="",C10=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B10&amp;C10," ",""))&amp;IF(E10&lt;&gt;"","-"&amp;RIGHT(E10,4),IF(J10&lt;&gt;"","-"&amp;RIGHT(J10,4),"")))</x:f>
+        <x:f>IF(AND(B10="",C10=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B10&amp;C10," ",""))&amp;IF(E10&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E10," ",""),4),IF(J10&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J10," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B10" s="16"/>
       <x:c r="C10" s="16"/>
@@ -753,7 +753,7 @@
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="16" t="str">
-        <x:f>IF(AND(B11="",C11=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B11&amp;C11," ",""))&amp;IF(E11&lt;&gt;"","-"&amp;RIGHT(E11,4),IF(J11&lt;&gt;"","-"&amp;RIGHT(J11,4),"")))</x:f>
+        <x:f>IF(AND(B11="",C11=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B11&amp;C11," ",""))&amp;IF(E11&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E11," ",""),4),IF(J11&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J11," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B11" s="16"/>
       <x:c r="C11" s="16"/>
@@ -779,7 +779,7 @@
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="16" t="str">
-        <x:f>IF(AND(B12="",C12=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B12&amp;C12," ",""))&amp;IF(E12&lt;&gt;"","-"&amp;RIGHT(E12,4),IF(J12&lt;&gt;"","-"&amp;RIGHT(J12,4),"")))</x:f>
+        <x:f>IF(AND(B12="",C12=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B12&amp;C12," ",""))&amp;IF(E12&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E12," ",""),4),IF(J12&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J12," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B12" s="16"/>
       <x:c r="C12" s="16"/>
@@ -805,7 +805,7 @@
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="16" t="str">
-        <x:f>IF(AND(B13="",C13=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B13&amp;C13," ",""))&amp;IF(E13&lt;&gt;"","-"&amp;RIGHT(E13,4),IF(J13&lt;&gt;"","-"&amp;RIGHT(J13,4),"")))</x:f>
+        <x:f>IF(AND(B13="",C13=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B13&amp;C13," ",""))&amp;IF(E13&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E13," ",""),4),IF(J13&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J13," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B13" s="16"/>
       <x:c r="C13" s="16"/>
@@ -831,7 +831,7 @@
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="16" t="str">
-        <x:f>IF(AND(B14="",C14=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B14&amp;C14," ",""))&amp;IF(E14&lt;&gt;"","-"&amp;RIGHT(E14,4),IF(J14&lt;&gt;"","-"&amp;RIGHT(J14,4),"")))</x:f>
+        <x:f>IF(AND(B14="",C14=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B14&amp;C14," ",""))&amp;IF(E14&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E14," ",""),4),IF(J14&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J14," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B14" s="16"/>
       <x:c r="C14" s="16"/>
@@ -857,7 +857,7 @@
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="16" t="str">
-        <x:f>IF(AND(B15="",C15=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B15&amp;C15," ",""))&amp;IF(E15&lt;&gt;"","-"&amp;RIGHT(E15,4),IF(J15&lt;&gt;"","-"&amp;RIGHT(J15,4),"")))</x:f>
+        <x:f>IF(AND(B15="",C15=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B15&amp;C15," ",""))&amp;IF(E15&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E15," ",""),4),IF(J15&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J15," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B15" s="16"/>
       <x:c r="C15" s="16"/>
@@ -883,7 +883,7 @@
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="16" t="str">
-        <x:f>IF(AND(B16="",C16=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B16&amp;C16," ",""))&amp;IF(E16&lt;&gt;"","-"&amp;RIGHT(E16,4),IF(J16&lt;&gt;"","-"&amp;RIGHT(J16,4),"")))</x:f>
+        <x:f>IF(AND(B16="",C16=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B16&amp;C16," ",""))&amp;IF(E16&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E16," ",""),4),IF(J16&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J16," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B16" s="16"/>
       <x:c r="C16" s="16"/>
@@ -909,7 +909,7 @@
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="16" t="str">
-        <x:f>IF(AND(B17="",C17=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B17&amp;C17," ",""))&amp;IF(E17&lt;&gt;"","-"&amp;RIGHT(E17,4),IF(J17&lt;&gt;"","-"&amp;RIGHT(J17,4),"")))</x:f>
+        <x:f>IF(AND(B17="",C17=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B17&amp;C17," ",""))&amp;IF(E17&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E17," ",""),4),IF(J17&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J17," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B17" s="16"/>
       <x:c r="C17" s="16"/>
@@ -935,7 +935,7 @@
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="16" t="str">
-        <x:f>IF(AND(B18="",C18=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B18&amp;C18," ",""))&amp;IF(E18&lt;&gt;"","-"&amp;RIGHT(E18,4),IF(J18&lt;&gt;"","-"&amp;RIGHT(J18,4),"")))</x:f>
+        <x:f>IF(AND(B18="",C18=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B18&amp;C18," ",""))&amp;IF(E18&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E18," ",""),4),IF(J18&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J18," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B18" s="16"/>
       <x:c r="C18" s="16"/>
@@ -961,7 +961,7 @@
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="16" t="str">
-        <x:f>IF(AND(B19="",C19=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B19&amp;C19," ",""))&amp;IF(E19&lt;&gt;"","-"&amp;RIGHT(E19,4),IF(J19&lt;&gt;"","-"&amp;RIGHT(J19,4),"")))</x:f>
+        <x:f>IF(AND(B19="",C19=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B19&amp;C19," ",""))&amp;IF(E19&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E19," ",""),4),IF(J19&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J19," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B19" s="16"/>
       <x:c r="C19" s="16"/>
@@ -987,7 +987,7 @@
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="16" t="str">
-        <x:f>IF(AND(B20="",C20=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B20&amp;C20," ",""))&amp;IF(E20&lt;&gt;"","-"&amp;RIGHT(E20,4),IF(J20&lt;&gt;"","-"&amp;RIGHT(J20,4),"")))</x:f>
+        <x:f>IF(AND(B20="",C20=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B20&amp;C20," ",""))&amp;IF(E20&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E20," ",""),4),IF(J20&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J20," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B20" s="16"/>
       <x:c r="C20" s="16"/>
@@ -1013,7 +1013,7 @@
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="16" t="str">
-        <x:f>IF(AND(B21="",C21=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B21&amp;C21," ",""))&amp;IF(E21&lt;&gt;"","-"&amp;RIGHT(E21,4),IF(J21&lt;&gt;"","-"&amp;RIGHT(J21,4),"")))</x:f>
+        <x:f>IF(AND(B21="",C21=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B21&amp;C21," ",""))&amp;IF(E21&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E21," ",""),4),IF(J21&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J21," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B21" s="16"/>
       <x:c r="C21" s="16"/>
@@ -1039,7 +1039,7 @@
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="16" t="str">
-        <x:f>IF(AND(B22="",C22=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B22&amp;C22," ",""))&amp;IF(E22&lt;&gt;"","-"&amp;RIGHT(E22,4),IF(J22&lt;&gt;"","-"&amp;RIGHT(J22,4),"")))</x:f>
+        <x:f>IF(AND(B22="",C22=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B22&amp;C22," ",""))&amp;IF(E22&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E22," ",""),4),IF(J22&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J22," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B22" s="16"/>
       <x:c r="C22" s="16"/>
@@ -1065,7 +1065,7 @@
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="16" t="str">
-        <x:f>IF(AND(B23="",C23=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B23&amp;C23," ",""))&amp;IF(E23&lt;&gt;"","-"&amp;RIGHT(E23,4),IF(J23&lt;&gt;"","-"&amp;RIGHT(J23,4),"")))</x:f>
+        <x:f>IF(AND(B23="",C23=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B23&amp;C23," ",""))&amp;IF(E23&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E23," ",""),4),IF(J23&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J23," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B23" s="16"/>
       <x:c r="C23" s="16"/>
@@ -1091,7 +1091,7 @@
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="16" t="str">
-        <x:f>IF(AND(B24="",C24=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B24&amp;C24," ",""))&amp;IF(E24&lt;&gt;"","-"&amp;RIGHT(E24,4),IF(J24&lt;&gt;"","-"&amp;RIGHT(J24,4),"")))</x:f>
+        <x:f>IF(AND(B24="",C24=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B24&amp;C24," ",""))&amp;IF(E24&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E24," ",""),4),IF(J24&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J24," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B24" s="16"/>
       <x:c r="C24" s="16"/>
@@ -1117,7 +1117,7 @@
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="16" t="str">
-        <x:f>IF(AND(B25="",C25=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B25&amp;C25," ",""))&amp;IF(E25&lt;&gt;"","-"&amp;RIGHT(E25,4),IF(J25&lt;&gt;"","-"&amp;RIGHT(J25,4),"")))</x:f>
+        <x:f>IF(AND(B25="",C25=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B25&amp;C25," ",""))&amp;IF(E25&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E25," ",""),4),IF(J25&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J25," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B25" s="16"/>
       <x:c r="C25" s="16"/>
@@ -1143,7 +1143,7 @@
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
       <x:c r="A26" s="16" t="str">
-        <x:f>IF(AND(B26="",C26=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B26&amp;C26," ",""))&amp;IF(E26&lt;&gt;"","-"&amp;RIGHT(E26,4),IF(J26&lt;&gt;"","-"&amp;RIGHT(J26,4),"")))</x:f>
+        <x:f>IF(AND(B26="",C26=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B26&amp;C26," ",""))&amp;IF(E26&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E26," ",""),4),IF(J26&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J26," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B26" s="16"/>
       <x:c r="C26" s="16"/>
@@ -1169,7 +1169,7 @@
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="16" t="str">
-        <x:f>IF(AND(B27="",C27=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B27&amp;C27," ",""))&amp;IF(E27&lt;&gt;"","-"&amp;RIGHT(E27,4),IF(J27&lt;&gt;"","-"&amp;RIGHT(J27,4),"")))</x:f>
+        <x:f>IF(AND(B27="",C27=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B27&amp;C27," ",""))&amp;IF(E27&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E27," ",""),4),IF(J27&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J27," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B27" s="16"/>
       <x:c r="C27" s="16"/>
@@ -1195,7 +1195,7 @@
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="16" t="str">
-        <x:f>IF(AND(B28="",C28=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B28&amp;C28," ",""))&amp;IF(E28&lt;&gt;"","-"&amp;RIGHT(E28,4),IF(J28&lt;&gt;"","-"&amp;RIGHT(J28,4),"")))</x:f>
+        <x:f>IF(AND(B28="",C28=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B28&amp;C28," ",""))&amp;IF(E28&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E28," ",""),4),IF(J28&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J28," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B28" s="16"/>
       <x:c r="C28" s="16"/>
@@ -1221,7 +1221,7 @@
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="16" t="str">
-        <x:f>IF(AND(B29="",C29=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B29&amp;C29," ",""))&amp;IF(E29&lt;&gt;"","-"&amp;RIGHT(E29,4),IF(J29&lt;&gt;"","-"&amp;RIGHT(J29,4),"")))</x:f>
+        <x:f>IF(AND(B29="",C29=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B29&amp;C29," ",""))&amp;IF(E29&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E29," ",""),4),IF(J29&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J29," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B29" s="16"/>
       <x:c r="C29" s="16"/>
@@ -1247,7 +1247,7 @@
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="16" t="str">
-        <x:f>IF(AND(B30="",C30=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B30&amp;C30," ",""))&amp;IF(E30&lt;&gt;"","-"&amp;RIGHT(E30,4),IF(J30&lt;&gt;"","-"&amp;RIGHT(J30,4),"")))</x:f>
+        <x:f>IF(AND(B30="",C30=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B30&amp;C30," ",""))&amp;IF(E30&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E30," ",""),4),IF(J30&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J30," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B30" s="16"/>
       <x:c r="C30" s="16"/>
@@ -1273,7 +1273,7 @@
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="16" t="str">
-        <x:f>IF(AND(B31="",C31=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B31&amp;C31," ",""))&amp;IF(E31&lt;&gt;"","-"&amp;RIGHT(E31,4),IF(J31&lt;&gt;"","-"&amp;RIGHT(J31,4),"")))</x:f>
+        <x:f>IF(AND(B31="",C31=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B31&amp;C31," ",""))&amp;IF(E31&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E31," ",""),4),IF(J31&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J31," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B31" s="16"/>
       <x:c r="C31" s="16"/>
@@ -1299,7 +1299,7 @@
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="16" t="str">
-        <x:f>IF(AND(B32="",C32=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B32&amp;C32," ",""))&amp;IF(E32&lt;&gt;"","-"&amp;RIGHT(E32,4),IF(J32&lt;&gt;"","-"&amp;RIGHT(J32,4),"")))</x:f>
+        <x:f>IF(AND(B32="",C32=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B32&amp;C32," ",""))&amp;IF(E32&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E32," ",""),4),IF(J32&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J32," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B32" s="16"/>
       <x:c r="C32" s="16"/>
@@ -1325,7 +1325,7 @@
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
       <x:c r="A33" s="16" t="str">
-        <x:f>IF(AND(B33="",C33=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B33&amp;C33," ",""))&amp;IF(E33&lt;&gt;"","-"&amp;RIGHT(E33,4),IF(J33&lt;&gt;"","-"&amp;RIGHT(J33,4),"")))</x:f>
+        <x:f>IF(AND(B33="",C33=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B33&amp;C33," ",""))&amp;IF(E33&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E33," ",""),4),IF(J33&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J33," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B33" s="16"/>
       <x:c r="C33" s="16"/>
@@ -1351,7 +1351,7 @@
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
       <x:c r="A34" s="16" t="str">
-        <x:f>IF(AND(B34="",C34=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B34&amp;C34," ",""))&amp;IF(E34&lt;&gt;"","-"&amp;RIGHT(E34,4),IF(J34&lt;&gt;"","-"&amp;RIGHT(J34,4),"")))</x:f>
+        <x:f>IF(AND(B34="",C34=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B34&amp;C34," ",""))&amp;IF(E34&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E34," ",""),4),IF(J34&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J34," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B34" s="16"/>
       <x:c r="C34" s="16"/>
@@ -1377,7 +1377,7 @@
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="16" t="str">
-        <x:f>IF(AND(B35="",C35=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B35&amp;C35," ",""))&amp;IF(E35&lt;&gt;"","-"&amp;RIGHT(E35,4),IF(J35&lt;&gt;"","-"&amp;RIGHT(J35,4),"")))</x:f>
+        <x:f>IF(AND(B35="",C35=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B35&amp;C35," ",""))&amp;IF(E35&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E35," ",""),4),IF(J35&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J35," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B35" s="16"/>
       <x:c r="C35" s="16"/>
@@ -1403,7 +1403,7 @@
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="16" t="str">
-        <x:f>IF(AND(B36="",C36=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B36&amp;C36," ",""))&amp;IF(E36&lt;&gt;"","-"&amp;RIGHT(E36,4),IF(J36&lt;&gt;"","-"&amp;RIGHT(J36,4),"")))</x:f>
+        <x:f>IF(AND(B36="",C36=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B36&amp;C36," ",""))&amp;IF(E36&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E36," ",""),4),IF(J36&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J36," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B36" s="16"/>
       <x:c r="C36" s="16"/>
@@ -1429,7 +1429,7 @@
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
       <x:c r="A37" s="16" t="str">
-        <x:f>IF(AND(B37="",C37=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B37&amp;C37," ",""))&amp;IF(E37&lt;&gt;"","-"&amp;RIGHT(E37,4),IF(J37&lt;&gt;"","-"&amp;RIGHT(J37,4),"")))</x:f>
+        <x:f>IF(AND(B37="",C37=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B37&amp;C37," ",""))&amp;IF(E37&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E37," ",""),4),IF(J37&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J37," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B37" s="16"/>
       <x:c r="C37" s="16"/>
@@ -1455,7 +1455,7 @@
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
       <x:c r="A38" s="16" t="str">
-        <x:f>IF(AND(B38="",C38=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B38&amp;C38," ",""))&amp;IF(E38&lt;&gt;"","-"&amp;RIGHT(E38,4),IF(J38&lt;&gt;"","-"&amp;RIGHT(J38,4),"")))</x:f>
+        <x:f>IF(AND(B38="",C38=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B38&amp;C38," ",""))&amp;IF(E38&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E38," ",""),4),IF(J38&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J38," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B38" s="16"/>
       <x:c r="C38" s="16"/>
@@ -1481,7 +1481,7 @@
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
       <x:c r="A39" s="16" t="str">
-        <x:f>IF(AND(B39="",C39=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B39&amp;C39," ",""))&amp;IF(E39&lt;&gt;"","-"&amp;RIGHT(E39,4),IF(J39&lt;&gt;"","-"&amp;RIGHT(J39,4),"")))</x:f>
+        <x:f>IF(AND(B39="",C39=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B39&amp;C39," ",""))&amp;IF(E39&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E39," ",""),4),IF(J39&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J39," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B39" s="16"/>
       <x:c r="C39" s="16"/>
@@ -1507,7 +1507,7 @@
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
       <x:c r="A40" s="16" t="str">
-        <x:f>IF(AND(B40="",C40=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B40&amp;C40," ",""))&amp;IF(E40&lt;&gt;"","-"&amp;RIGHT(E40,4),IF(J40&lt;&gt;"","-"&amp;RIGHT(J40,4),"")))</x:f>
+        <x:f>IF(AND(B40="",C40=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B40&amp;C40," ",""))&amp;IF(E40&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E40," ",""),4),IF(J40&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J40," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B40" s="16"/>
       <x:c r="C40" s="16"/>
@@ -1533,7 +1533,7 @@
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
       <x:c r="A41" s="16" t="str">
-        <x:f>IF(AND(B41="",C41=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B41&amp;C41," ",""))&amp;IF(E41&lt;&gt;"","-"&amp;RIGHT(E41,4),IF(J41&lt;&gt;"","-"&amp;RIGHT(J41,4),"")))</x:f>
+        <x:f>IF(AND(B41="",C41=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B41&amp;C41," ",""))&amp;IF(E41&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E41," ",""),4),IF(J41&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J41," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B41" s="16"/>
       <x:c r="C41" s="16"/>
@@ -1559,7 +1559,7 @@
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
       <x:c r="A42" s="16" t="str">
-        <x:f>IF(AND(B42="",C42=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B42&amp;C42," ",""))&amp;IF(E42&lt;&gt;"","-"&amp;RIGHT(E42,4),IF(J42&lt;&gt;"","-"&amp;RIGHT(J42,4),"")))</x:f>
+        <x:f>IF(AND(B42="",C42=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B42&amp;C42," ",""))&amp;IF(E42&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E42," ",""),4),IF(J42&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J42," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B42" s="16"/>
       <x:c r="C42" s="16"/>
@@ -1585,7 +1585,7 @@
     </x:row>
     <x:row r="43" ht="15" hidden="0" customHeight="1">
       <x:c r="A43" s="16" t="str">
-        <x:f>IF(AND(B43="",C43=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B43&amp;C43," ",""))&amp;IF(E43&lt;&gt;"","-"&amp;RIGHT(E43,4),IF(J43&lt;&gt;"","-"&amp;RIGHT(J43,4),"")))</x:f>
+        <x:f>IF(AND(B43="",C43=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B43&amp;C43," ",""))&amp;IF(E43&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E43," ",""),4),IF(J43&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J43," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B43" s="16"/>
       <x:c r="C43" s="16"/>
@@ -1611,7 +1611,7 @@
     </x:row>
     <x:row r="44" ht="15" hidden="0" customHeight="1">
       <x:c r="A44" s="16" t="str">
-        <x:f>IF(AND(B44="",C44=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B44&amp;C44," ",""))&amp;IF(E44&lt;&gt;"","-"&amp;RIGHT(E44,4),IF(J44&lt;&gt;"","-"&amp;RIGHT(J44,4),"")))</x:f>
+        <x:f>IF(AND(B44="",C44=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B44&amp;C44," ",""))&amp;IF(E44&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E44," ",""),4),IF(J44&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J44," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B44" s="16"/>
       <x:c r="C44" s="16"/>
@@ -1637,7 +1637,7 @@
     </x:row>
     <x:row r="45" ht="15" hidden="0" customHeight="1">
       <x:c r="A45" s="16" t="str">
-        <x:f>IF(AND(B45="",C45=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B45&amp;C45," ",""))&amp;IF(E45&lt;&gt;"","-"&amp;RIGHT(E45,4),IF(J45&lt;&gt;"","-"&amp;RIGHT(J45,4),"")))</x:f>
+        <x:f>IF(AND(B45="",C45=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B45&amp;C45," ",""))&amp;IF(E45&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E45," ",""),4),IF(J45&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J45," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B45" s="16"/>
       <x:c r="C45" s="16"/>
@@ -1663,7 +1663,7 @@
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
       <x:c r="A46" s="16" t="str">
-        <x:f>IF(AND(B46="",C46=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B46&amp;C46," ",""))&amp;IF(E46&lt;&gt;"","-"&amp;RIGHT(E46,4),IF(J46&lt;&gt;"","-"&amp;RIGHT(J46,4),"")))</x:f>
+        <x:f>IF(AND(B46="",C46=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B46&amp;C46," ",""))&amp;IF(E46&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E46," ",""),4),IF(J46&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J46," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B46" s="16"/>
       <x:c r="C46" s="16"/>
@@ -1689,7 +1689,7 @@
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
       <x:c r="A47" s="16" t="str">
-        <x:f>IF(AND(B47="",C47=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B47&amp;C47," ",""))&amp;IF(E47&lt;&gt;"","-"&amp;RIGHT(E47,4),IF(J47&lt;&gt;"","-"&amp;RIGHT(J47,4),"")))</x:f>
+        <x:f>IF(AND(B47="",C47=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B47&amp;C47," ",""))&amp;IF(E47&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E47," ",""),4),IF(J47&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J47," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B47" s="16"/>
       <x:c r="C47" s="16"/>
@@ -1715,7 +1715,7 @@
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
       <x:c r="A48" s="16" t="str">
-        <x:f>IF(AND(B48="",C48=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B48&amp;C48," ",""))&amp;IF(E48&lt;&gt;"","-"&amp;RIGHT(E48,4),IF(J48&lt;&gt;"","-"&amp;RIGHT(J48,4),"")))</x:f>
+        <x:f>IF(AND(B48="",C48=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B48&amp;C48," ",""))&amp;IF(E48&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E48," ",""),4),IF(J48&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J48," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B48" s="16"/>
       <x:c r="C48" s="16"/>
@@ -1741,7 +1741,7 @@
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
       <x:c r="A49" s="16" t="str">
-        <x:f>IF(AND(B49="",C49=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B49&amp;C49," ",""))&amp;IF(E49&lt;&gt;"","-"&amp;RIGHT(E49,4),IF(J49&lt;&gt;"","-"&amp;RIGHT(J49,4),"")))</x:f>
+        <x:f>IF(AND(B49="",C49=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B49&amp;C49," ",""))&amp;IF(E49&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E49," ",""),4),IF(J49&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J49," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B49" s="16"/>
       <x:c r="C49" s="16"/>
@@ -1767,7 +1767,7 @@
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
       <x:c r="A50" s="16" t="str">
-        <x:f>IF(AND(B50="",C50=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B50&amp;C50," ",""))&amp;IF(E50&lt;&gt;"","-"&amp;RIGHT(E50,4),IF(J50&lt;&gt;"","-"&amp;RIGHT(J50,4),"")))</x:f>
+        <x:f>IF(AND(B50="",C50=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B50&amp;C50," ",""))&amp;IF(E50&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E50," ",""),4),IF(J50&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J50," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B50" s="16"/>
       <x:c r="C50" s="16"/>
@@ -1793,7 +1793,7 @@
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
       <x:c r="A51" s="16" t="str">
-        <x:f>IF(AND(B51="",C51=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B51&amp;C51," ",""))&amp;IF(E51&lt;&gt;"","-"&amp;RIGHT(E51,4),IF(J51&lt;&gt;"","-"&amp;RIGHT(J51,4),"")))</x:f>
+        <x:f>IF(AND(B51="",C51=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B51&amp;C51," ",""))&amp;IF(E51&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E51," ",""),4),IF(J51&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J51," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B51" s="16"/>
       <x:c r="C51" s="16"/>
@@ -1819,7 +1819,7 @@
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
       <x:c r="A52" s="16" t="str">
-        <x:f>IF(AND(B52="",C52=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B52&amp;C52," ",""))&amp;IF(E52&lt;&gt;"","-"&amp;RIGHT(E52,4),IF(J52&lt;&gt;"","-"&amp;RIGHT(J52,4),"")))</x:f>
+        <x:f>IF(AND(B52="",C52=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B52&amp;C52," ",""))&amp;IF(E52&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E52," ",""),4),IF(J52&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J52," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B52" s="16"/>
       <x:c r="C52" s="16"/>
@@ -1845,7 +1845,7 @@
     </x:row>
     <x:row r="53" ht="15" hidden="0" customHeight="1">
       <x:c r="A53" s="16" t="str">
-        <x:f>IF(AND(B53="",C53=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B53&amp;C53," ",""))&amp;IF(E53&lt;&gt;"","-"&amp;RIGHT(E53,4),IF(J53&lt;&gt;"","-"&amp;RIGHT(J53,4),"")))</x:f>
+        <x:f>IF(AND(B53="",C53=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B53&amp;C53," ",""))&amp;IF(E53&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E53," ",""),4),IF(J53&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J53," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B53" s="16"/>
       <x:c r="C53" s="16"/>
@@ -1871,7 +1871,7 @@
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
       <x:c r="A54" s="16" t="str">
-        <x:f>IF(AND(B54="",C54=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B54&amp;C54," ",""))&amp;IF(E54&lt;&gt;"","-"&amp;RIGHT(E54,4),IF(J54&lt;&gt;"","-"&amp;RIGHT(J54,4),"")))</x:f>
+        <x:f>IF(AND(B54="",C54=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B54&amp;C54," ",""))&amp;IF(E54&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E54," ",""),4),IF(J54&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J54," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B54" s="16"/>
       <x:c r="C54" s="16"/>
@@ -1897,7 +1897,7 @@
     </x:row>
     <x:row r="55" ht="15" hidden="0" customHeight="1">
       <x:c r="A55" s="16" t="str">
-        <x:f>IF(AND(B55="",C55=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B55&amp;C55," ",""))&amp;IF(E55&lt;&gt;"","-"&amp;RIGHT(E55,4),IF(J55&lt;&gt;"","-"&amp;RIGHT(J55,4),"")))</x:f>
+        <x:f>IF(AND(B55="",C55=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B55&amp;C55," ",""))&amp;IF(E55&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E55," ",""),4),IF(J55&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J55," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B55" s="16"/>
       <x:c r="C55" s="16"/>
@@ -1923,7 +1923,7 @@
     </x:row>
     <x:row r="56" ht="15" hidden="0" customHeight="1">
       <x:c r="A56" s="16" t="str">
-        <x:f>IF(AND(B56="",C56=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B56&amp;C56," ",""))&amp;IF(E56&lt;&gt;"","-"&amp;RIGHT(E56,4),IF(J56&lt;&gt;"","-"&amp;RIGHT(J56,4),"")))</x:f>
+        <x:f>IF(AND(B56="",C56=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B56&amp;C56," ",""))&amp;IF(E56&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E56," ",""),4),IF(J56&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J56," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B56" s="16"/>
       <x:c r="C56" s="16"/>
@@ -1949,7 +1949,7 @@
     </x:row>
     <x:row r="57" ht="15" hidden="0" customHeight="1">
       <x:c r="A57" s="16" t="str">
-        <x:f>IF(AND(B57="",C57=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B57&amp;C57," ",""))&amp;IF(E57&lt;&gt;"","-"&amp;RIGHT(E57,4),IF(J57&lt;&gt;"","-"&amp;RIGHT(J57,4),"")))</x:f>
+        <x:f>IF(AND(B57="",C57=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B57&amp;C57," ",""))&amp;IF(E57&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E57," ",""),4),IF(J57&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J57," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B57" s="16"/>
       <x:c r="C57" s="16"/>
@@ -1975,7 +1975,7 @@
     </x:row>
     <x:row r="58" ht="15" hidden="0" customHeight="1">
       <x:c r="A58" s="16" t="str">
-        <x:f>IF(AND(B58="",C58=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B58&amp;C58," ",""))&amp;IF(E58&lt;&gt;"","-"&amp;RIGHT(E58,4),IF(J58&lt;&gt;"","-"&amp;RIGHT(J58,4),"")))</x:f>
+        <x:f>IF(AND(B58="",C58=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B58&amp;C58," ",""))&amp;IF(E58&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E58," ",""),4),IF(J58&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J58," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B58" s="16"/>
       <x:c r="C58" s="16"/>
@@ -2001,7 +2001,7 @@
     </x:row>
     <x:row r="59" ht="15" hidden="0" customHeight="1">
       <x:c r="A59" s="16" t="str">
-        <x:f>IF(AND(B59="",C59=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B59&amp;C59," ",""))&amp;IF(E59&lt;&gt;"","-"&amp;RIGHT(E59,4),IF(J59&lt;&gt;"","-"&amp;RIGHT(J59,4),"")))</x:f>
+        <x:f>IF(AND(B59="",C59=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B59&amp;C59," ",""))&amp;IF(E59&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E59," ",""),4),IF(J59&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J59," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B59" s="16"/>
       <x:c r="C59" s="16"/>
@@ -2027,7 +2027,7 @@
     </x:row>
     <x:row r="60" ht="15" hidden="0" customHeight="1">
       <x:c r="A60" s="16" t="str">
-        <x:f>IF(AND(B60="",C60=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B60&amp;C60," ",""))&amp;IF(E60&lt;&gt;"","-"&amp;RIGHT(E60,4),IF(J60&lt;&gt;"","-"&amp;RIGHT(J60,4),"")))</x:f>
+        <x:f>IF(AND(B60="",C60=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B60&amp;C60," ",""))&amp;IF(E60&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E60," ",""),4),IF(J60&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J60," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B60" s="16"/>
       <x:c r="C60" s="16"/>
@@ -2053,7 +2053,7 @@
     </x:row>
     <x:row r="61" ht="15" hidden="0" customHeight="1">
       <x:c r="A61" s="16" t="str">
-        <x:f>IF(AND(B61="",C61=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B61&amp;C61," ",""))&amp;IF(E61&lt;&gt;"","-"&amp;RIGHT(E61,4),IF(J61&lt;&gt;"","-"&amp;RIGHT(J61,4),"")))</x:f>
+        <x:f>IF(AND(B61="",C61=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B61&amp;C61," ",""))&amp;IF(E61&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E61," ",""),4),IF(J61&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J61," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B61" s="16"/>
       <x:c r="C61" s="16"/>
@@ -2079,7 +2079,7 @@
     </x:row>
     <x:row r="62" ht="15" hidden="0" customHeight="1">
       <x:c r="A62" s="16" t="str">
-        <x:f>IF(AND(B62="",C62=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B62&amp;C62," ",""))&amp;IF(E62&lt;&gt;"","-"&amp;RIGHT(E62,4),IF(J62&lt;&gt;"","-"&amp;RIGHT(J62,4),"")))</x:f>
+        <x:f>IF(AND(B62="",C62=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B62&amp;C62," ",""))&amp;IF(E62&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E62," ",""),4),IF(J62&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J62," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B62" s="16"/>
       <x:c r="C62" s="16"/>
@@ -2105,7 +2105,7 @@
     </x:row>
     <x:row r="63" ht="15" hidden="0" customHeight="1">
       <x:c r="A63" s="16" t="str">
-        <x:f>IF(AND(B63="",C63=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B63&amp;C63," ",""))&amp;IF(E63&lt;&gt;"","-"&amp;RIGHT(E63,4),IF(J63&lt;&gt;"","-"&amp;RIGHT(J63,4),"")))</x:f>
+        <x:f>IF(AND(B63="",C63=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B63&amp;C63," ",""))&amp;IF(E63&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E63," ",""),4),IF(J63&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J63," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B63" s="16"/>
       <x:c r="C63" s="16"/>
@@ -2131,7 +2131,7 @@
     </x:row>
     <x:row r="64" ht="15" hidden="0" customHeight="1">
       <x:c r="A64" s="16" t="str">
-        <x:f>IF(AND(B64="",C64=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B64&amp;C64," ",""))&amp;IF(E64&lt;&gt;"","-"&amp;RIGHT(E64,4),IF(J64&lt;&gt;"","-"&amp;RIGHT(J64,4),"")))</x:f>
+        <x:f>IF(AND(B64="",C64=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B64&amp;C64," ",""))&amp;IF(E64&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E64," ",""),4),IF(J64&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J64," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B64" s="16"/>
       <x:c r="C64" s="16"/>
@@ -2157,7 +2157,7 @@
     </x:row>
     <x:row r="65" ht="15" hidden="0" customHeight="1">
       <x:c r="A65" s="16" t="str">
-        <x:f>IF(AND(B65="",C65=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B65&amp;C65," ",""))&amp;IF(E65&lt;&gt;"","-"&amp;RIGHT(E65,4),IF(J65&lt;&gt;"","-"&amp;RIGHT(J65,4),"")))</x:f>
+        <x:f>IF(AND(B65="",C65=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B65&amp;C65," ",""))&amp;IF(E65&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E65," ",""),4),IF(J65&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J65," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B65" s="16"/>
       <x:c r="C65" s="16"/>
@@ -2183,7 +2183,7 @@
     </x:row>
     <x:row r="66" ht="15" hidden="0" customHeight="1">
       <x:c r="A66" s="16" t="str">
-        <x:f>IF(AND(B66="",C66=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B66&amp;C66," ",""))&amp;IF(E66&lt;&gt;"","-"&amp;RIGHT(E66,4),IF(J66&lt;&gt;"","-"&amp;RIGHT(J66,4),"")))</x:f>
+        <x:f>IF(AND(B66="",C66=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B66&amp;C66," ",""))&amp;IF(E66&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E66," ",""),4),IF(J66&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J66," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B66" s="16"/>
       <x:c r="C66" s="16"/>
@@ -2209,7 +2209,7 @@
     </x:row>
     <x:row r="67" ht="15" hidden="0" customHeight="1">
       <x:c r="A67" s="16" t="str">
-        <x:f>IF(AND(B67="",C67=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B67&amp;C67," ",""))&amp;IF(E67&lt;&gt;"","-"&amp;RIGHT(E67,4),IF(J67&lt;&gt;"","-"&amp;RIGHT(J67,4),"")))</x:f>
+        <x:f>IF(AND(B67="",C67=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B67&amp;C67," ",""))&amp;IF(E67&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E67," ",""),4),IF(J67&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J67," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B67" s="16"/>
       <x:c r="C67" s="16"/>
@@ -2235,7 +2235,7 @@
     </x:row>
     <x:row r="68" ht="15" hidden="0" customHeight="1">
       <x:c r="A68" s="16" t="str">
-        <x:f>IF(AND(B68="",C68=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B68&amp;C68," ",""))&amp;IF(E68&lt;&gt;"","-"&amp;RIGHT(E68,4),IF(J68&lt;&gt;"","-"&amp;RIGHT(J68,4),"")))</x:f>
+        <x:f>IF(AND(B68="",C68=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B68&amp;C68," ",""))&amp;IF(E68&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E68," ",""),4),IF(J68&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J68," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B68" s="16"/>
       <x:c r="C68" s="16"/>
@@ -2261,7 +2261,7 @@
     </x:row>
     <x:row r="69" ht="15" hidden="0" customHeight="1">
       <x:c r="A69" s="16" t="str">
-        <x:f>IF(AND(B69="",C69=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B69&amp;C69," ",""))&amp;IF(E69&lt;&gt;"","-"&amp;RIGHT(E69,4),IF(J69&lt;&gt;"","-"&amp;RIGHT(J69,4),"")))</x:f>
+        <x:f>IF(AND(B69="",C69=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B69&amp;C69," ",""))&amp;IF(E69&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E69," ",""),4),IF(J69&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J69," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B69" s="16"/>
       <x:c r="C69" s="16"/>
@@ -2287,7 +2287,7 @@
     </x:row>
     <x:row r="70" ht="15" hidden="0" customHeight="1">
       <x:c r="A70" s="16" t="str">
-        <x:f>IF(AND(B70="",C70=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B70&amp;C70," ",""))&amp;IF(E70&lt;&gt;"","-"&amp;RIGHT(E70,4),IF(J70&lt;&gt;"","-"&amp;RIGHT(J70,4),"")))</x:f>
+        <x:f>IF(AND(B70="",C70=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B70&amp;C70," ",""))&amp;IF(E70&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E70," ",""),4),IF(J70&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J70," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B70" s="16"/>
       <x:c r="C70" s="16"/>
@@ -2313,7 +2313,7 @@
     </x:row>
     <x:row r="71" ht="15" hidden="0" customHeight="1">
       <x:c r="A71" s="16" t="str">
-        <x:f>IF(AND(B71="",C71=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B71&amp;C71," ",""))&amp;IF(E71&lt;&gt;"","-"&amp;RIGHT(E71,4),IF(J71&lt;&gt;"","-"&amp;RIGHT(J71,4),"")))</x:f>
+        <x:f>IF(AND(B71="",C71=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B71&amp;C71," ",""))&amp;IF(E71&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E71," ",""),4),IF(J71&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J71," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B71" s="16"/>
       <x:c r="C71" s="16"/>
@@ -2339,7 +2339,7 @@
     </x:row>
     <x:row r="72" ht="15" hidden="0" customHeight="1">
       <x:c r="A72" s="16" t="str">
-        <x:f>IF(AND(B72="",C72=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B72&amp;C72," ",""))&amp;IF(E72&lt;&gt;"","-"&amp;RIGHT(E72,4),IF(J72&lt;&gt;"","-"&amp;RIGHT(J72,4),"")))</x:f>
+        <x:f>IF(AND(B72="",C72=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B72&amp;C72," ",""))&amp;IF(E72&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E72," ",""),4),IF(J72&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J72," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B72" s="16"/>
       <x:c r="C72" s="16"/>
@@ -2365,7 +2365,7 @@
     </x:row>
     <x:row r="73" ht="15" hidden="0" customHeight="1">
       <x:c r="A73" s="16" t="str">
-        <x:f>IF(AND(B73="",C73=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B73&amp;C73," ",""))&amp;IF(E73&lt;&gt;"","-"&amp;RIGHT(E73,4),IF(J73&lt;&gt;"","-"&amp;RIGHT(J73,4),"")))</x:f>
+        <x:f>IF(AND(B73="",C73=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B73&amp;C73," ",""))&amp;IF(E73&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E73," ",""),4),IF(J73&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J73," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B73" s="16"/>
       <x:c r="C73" s="16"/>
@@ -2391,7 +2391,7 @@
     </x:row>
     <x:row r="74" ht="15" hidden="0" customHeight="1">
       <x:c r="A74" s="16" t="str">
-        <x:f>IF(AND(B74="",C74=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B74&amp;C74," ",""))&amp;IF(E74&lt;&gt;"","-"&amp;RIGHT(E74,4),IF(J74&lt;&gt;"","-"&amp;RIGHT(J74,4),"")))</x:f>
+        <x:f>IF(AND(B74="",C74=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B74&amp;C74," ",""))&amp;IF(E74&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E74," ",""),4),IF(J74&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J74," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B74" s="16"/>
       <x:c r="C74" s="16"/>
@@ -2417,7 +2417,7 @@
     </x:row>
     <x:row r="75" ht="15" hidden="0" customHeight="1">
       <x:c r="A75" s="16" t="str">
-        <x:f>IF(AND(B75="",C75=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B75&amp;C75," ",""))&amp;IF(E75&lt;&gt;"","-"&amp;RIGHT(E75,4),IF(J75&lt;&gt;"","-"&amp;RIGHT(J75,4),"")))</x:f>
+        <x:f>IF(AND(B75="",C75=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B75&amp;C75," ",""))&amp;IF(E75&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E75," ",""),4),IF(J75&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J75," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B75" s="16"/>
       <x:c r="C75" s="16"/>
@@ -2443,7 +2443,7 @@
     </x:row>
     <x:row r="76" ht="15" hidden="0" customHeight="1">
       <x:c r="A76" s="16" t="str">
-        <x:f>IF(AND(B76="",C76=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B76&amp;C76," ",""))&amp;IF(E76&lt;&gt;"","-"&amp;RIGHT(E76,4),IF(J76&lt;&gt;"","-"&amp;RIGHT(J76,4),"")))</x:f>
+        <x:f>IF(AND(B76="",C76=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B76&amp;C76," ",""))&amp;IF(E76&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E76," ",""),4),IF(J76&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J76," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B76" s="16"/>
       <x:c r="C76" s="16"/>
@@ -2469,7 +2469,7 @@
     </x:row>
     <x:row r="77" ht="15" hidden="0" customHeight="1">
       <x:c r="A77" s="16" t="str">
-        <x:f>IF(AND(B77="",C77=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B77&amp;C77," ",""))&amp;IF(E77&lt;&gt;"","-"&amp;RIGHT(E77,4),IF(J77&lt;&gt;"","-"&amp;RIGHT(J77,4),"")))</x:f>
+        <x:f>IF(AND(B77="",C77=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B77&amp;C77," ",""))&amp;IF(E77&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E77," ",""),4),IF(J77&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J77," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B77" s="16"/>
       <x:c r="C77" s="16"/>
@@ -2495,7 +2495,7 @@
     </x:row>
     <x:row r="78" ht="15" hidden="0" customHeight="1">
       <x:c r="A78" s="16" t="str">
-        <x:f>IF(AND(B78="",C78=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B78&amp;C78," ",""))&amp;IF(E78&lt;&gt;"","-"&amp;RIGHT(E78,4),IF(J78&lt;&gt;"","-"&amp;RIGHT(J78,4),"")))</x:f>
+        <x:f>IF(AND(B78="",C78=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B78&amp;C78," ",""))&amp;IF(E78&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E78," ",""),4),IF(J78&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J78," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B78" s="16"/>
       <x:c r="C78" s="16"/>
@@ -2521,7 +2521,7 @@
     </x:row>
     <x:row r="79" ht="15" hidden="0" customHeight="1">
       <x:c r="A79" s="16" t="str">
-        <x:f>IF(AND(B79="",C79=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B79&amp;C79," ",""))&amp;IF(E79&lt;&gt;"","-"&amp;RIGHT(E79,4),IF(J79&lt;&gt;"","-"&amp;RIGHT(J79,4),"")))</x:f>
+        <x:f>IF(AND(B79="",C79=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B79&amp;C79," ",""))&amp;IF(E79&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E79," ",""),4),IF(J79&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J79," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B79" s="16"/>
       <x:c r="C79" s="16"/>
@@ -2547,7 +2547,7 @@
     </x:row>
     <x:row r="80" ht="15" hidden="0" customHeight="1">
       <x:c r="A80" s="16" t="str">
-        <x:f>IF(AND(B80="",C80=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B80&amp;C80," ",""))&amp;IF(E80&lt;&gt;"","-"&amp;RIGHT(E80,4),IF(J80&lt;&gt;"","-"&amp;RIGHT(J80,4),"")))</x:f>
+        <x:f>IF(AND(B80="",C80=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B80&amp;C80," ",""))&amp;IF(E80&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E80," ",""),4),IF(J80&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J80," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B80" s="16"/>
       <x:c r="C80" s="16"/>
@@ -2573,7 +2573,7 @@
     </x:row>
     <x:row r="81" ht="15" hidden="0" customHeight="1">
       <x:c r="A81" s="16" t="str">
-        <x:f>IF(AND(B81="",C81=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B81&amp;C81," ",""))&amp;IF(E81&lt;&gt;"","-"&amp;RIGHT(E81,4),IF(J81&lt;&gt;"","-"&amp;RIGHT(J81,4),"")))</x:f>
+        <x:f>IF(AND(B81="",C81=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B81&amp;C81," ",""))&amp;IF(E81&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E81," ",""),4),IF(J81&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J81," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B81" s="16"/>
       <x:c r="C81" s="16"/>
@@ -2599,7 +2599,7 @@
     </x:row>
     <x:row r="82" ht="15" hidden="0" customHeight="1">
       <x:c r="A82" s="16" t="str">
-        <x:f>IF(AND(B82="",C82=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B82&amp;C82," ",""))&amp;IF(E82&lt;&gt;"","-"&amp;RIGHT(E82,4),IF(J82&lt;&gt;"","-"&amp;RIGHT(J82,4),"")))</x:f>
+        <x:f>IF(AND(B82="",C82=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B82&amp;C82," ",""))&amp;IF(E82&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E82," ",""),4),IF(J82&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J82," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B82" s="16"/>
       <x:c r="C82" s="16"/>
@@ -2625,7 +2625,7 @@
     </x:row>
     <x:row r="83" ht="15" hidden="0" customHeight="1">
       <x:c r="A83" s="16" t="str">
-        <x:f>IF(AND(B83="",C83=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B83&amp;C83," ",""))&amp;IF(E83&lt;&gt;"","-"&amp;RIGHT(E83,4),IF(J83&lt;&gt;"","-"&amp;RIGHT(J83,4),"")))</x:f>
+        <x:f>IF(AND(B83="",C83=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B83&amp;C83," ",""))&amp;IF(E83&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E83," ",""),4),IF(J83&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J83," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B83" s="16"/>
       <x:c r="C83" s="16"/>
@@ -2651,7 +2651,7 @@
     </x:row>
     <x:row r="84" ht="15" hidden="0" customHeight="1">
       <x:c r="A84" s="16" t="str">
-        <x:f>IF(AND(B84="",C84=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B84&amp;C84," ",""))&amp;IF(E84&lt;&gt;"","-"&amp;RIGHT(E84,4),IF(J84&lt;&gt;"","-"&amp;RIGHT(J84,4),"")))</x:f>
+        <x:f>IF(AND(B84="",C84=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B84&amp;C84," ",""))&amp;IF(E84&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E84," ",""),4),IF(J84&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J84," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B84" s="16"/>
       <x:c r="C84" s="16"/>
@@ -2677,7 +2677,7 @@
     </x:row>
     <x:row r="85" ht="15" hidden="0" customHeight="1">
       <x:c r="A85" s="16" t="str">
-        <x:f>IF(AND(B85="",C85=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B85&amp;C85," ",""))&amp;IF(E85&lt;&gt;"","-"&amp;RIGHT(E85,4),IF(J85&lt;&gt;"","-"&amp;RIGHT(J85,4),"")))</x:f>
+        <x:f>IF(AND(B85="",C85=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B85&amp;C85," ",""))&amp;IF(E85&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E85," ",""),4),IF(J85&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J85," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B85" s="16"/>
       <x:c r="C85" s="16"/>
@@ -2703,7 +2703,7 @@
     </x:row>
     <x:row r="86" ht="15" hidden="0" customHeight="1">
       <x:c r="A86" s="16" t="str">
-        <x:f>IF(AND(B86="",C86=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B86&amp;C86," ",""))&amp;IF(E86&lt;&gt;"","-"&amp;RIGHT(E86,4),IF(J86&lt;&gt;"","-"&amp;RIGHT(J86,4),"")))</x:f>
+        <x:f>IF(AND(B86="",C86=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B86&amp;C86," ",""))&amp;IF(E86&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E86," ",""),4),IF(J86&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J86," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B86" s="16"/>
       <x:c r="C86" s="16"/>
@@ -2729,7 +2729,7 @@
     </x:row>
     <x:row r="87" ht="15" hidden="0" customHeight="1">
       <x:c r="A87" s="16" t="str">
-        <x:f>IF(AND(B87="",C87=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B87&amp;C87," ",""))&amp;IF(E87&lt;&gt;"","-"&amp;RIGHT(E87,4),IF(J87&lt;&gt;"","-"&amp;RIGHT(J87,4),"")))</x:f>
+        <x:f>IF(AND(B87="",C87=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B87&amp;C87," ",""))&amp;IF(E87&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E87," ",""),4),IF(J87&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J87," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B87" s="16"/>
       <x:c r="C87" s="16"/>
@@ -2755,7 +2755,7 @@
     </x:row>
     <x:row r="88" ht="15" hidden="0" customHeight="1">
       <x:c r="A88" s="16" t="str">
-        <x:f>IF(AND(B88="",C88=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B88&amp;C88," ",""))&amp;IF(E88&lt;&gt;"","-"&amp;RIGHT(E88,4),IF(J88&lt;&gt;"","-"&amp;RIGHT(J88,4),"")))</x:f>
+        <x:f>IF(AND(B88="",C88=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B88&amp;C88," ",""))&amp;IF(E88&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E88," ",""),4),IF(J88&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J88," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B88" s="16"/>
       <x:c r="C88" s="16"/>
@@ -2781,7 +2781,7 @@
     </x:row>
     <x:row r="89" ht="15" hidden="0" customHeight="1">
       <x:c r="A89" s="16" t="str">
-        <x:f>IF(AND(B89="",C89=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B89&amp;C89," ",""))&amp;IF(E89&lt;&gt;"","-"&amp;RIGHT(E89,4),IF(J89&lt;&gt;"","-"&amp;RIGHT(J89,4),"")))</x:f>
+        <x:f>IF(AND(B89="",C89=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B89&amp;C89," ",""))&amp;IF(E89&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E89," ",""),4),IF(J89&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J89," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B89" s="16"/>
       <x:c r="C89" s="16"/>
@@ -2807,7 +2807,7 @@
     </x:row>
     <x:row r="90" ht="15" hidden="0" customHeight="1">
       <x:c r="A90" s="16" t="str">
-        <x:f>IF(AND(B90="",C90=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B90&amp;C90," ",""))&amp;IF(E90&lt;&gt;"","-"&amp;RIGHT(E90,4),IF(J90&lt;&gt;"","-"&amp;RIGHT(J90,4),"")))</x:f>
+        <x:f>IF(AND(B90="",C90=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B90&amp;C90," ",""))&amp;IF(E90&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E90," ",""),4),IF(J90&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J90," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B90" s="16"/>
       <x:c r="C90" s="16"/>
@@ -2833,7 +2833,7 @@
     </x:row>
     <x:row r="91" ht="15" hidden="0" customHeight="1">
       <x:c r="A91" s="16" t="str">
-        <x:f>IF(AND(B91="",C91=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B91&amp;C91," ",""))&amp;IF(E91&lt;&gt;"","-"&amp;RIGHT(E91,4),IF(J91&lt;&gt;"","-"&amp;RIGHT(J91,4),"")))</x:f>
+        <x:f>IF(AND(B91="",C91=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B91&amp;C91," ",""))&amp;IF(E91&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E91," ",""),4),IF(J91&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J91," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B91" s="16"/>
       <x:c r="C91" s="16"/>
@@ -2859,7 +2859,7 @@
     </x:row>
     <x:row r="92" ht="15" hidden="0" customHeight="1">
       <x:c r="A92" s="16" t="str">
-        <x:f>IF(AND(B92="",C92=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B92&amp;C92," ",""))&amp;IF(E92&lt;&gt;"","-"&amp;RIGHT(E92,4),IF(J92&lt;&gt;"","-"&amp;RIGHT(J92,4),"")))</x:f>
+        <x:f>IF(AND(B92="",C92=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B92&amp;C92," ",""))&amp;IF(E92&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E92," ",""),4),IF(J92&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J92," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B92" s="16"/>
       <x:c r="C92" s="16"/>
@@ -2885,7 +2885,7 @@
     </x:row>
     <x:row r="93" ht="15" hidden="0" customHeight="1">
       <x:c r="A93" s="16" t="str">
-        <x:f>IF(AND(B93="",C93=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B93&amp;C93," ",""))&amp;IF(E93&lt;&gt;"","-"&amp;RIGHT(E93,4),IF(J93&lt;&gt;"","-"&amp;RIGHT(J93,4),"")))</x:f>
+        <x:f>IF(AND(B93="",C93=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B93&amp;C93," ",""))&amp;IF(E93&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E93," ",""),4),IF(J93&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J93," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B93" s="16"/>
       <x:c r="C93" s="16"/>
@@ -2911,7 +2911,7 @@
     </x:row>
     <x:row r="94" ht="15" hidden="0" customHeight="1">
       <x:c r="A94" s="16" t="str">
-        <x:f>IF(AND(B94="",C94=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B94&amp;C94," ",""))&amp;IF(E94&lt;&gt;"","-"&amp;RIGHT(E94,4),IF(J94&lt;&gt;"","-"&amp;RIGHT(J94,4),"")))</x:f>
+        <x:f>IF(AND(B94="",C94=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B94&amp;C94," ",""))&amp;IF(E94&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E94," ",""),4),IF(J94&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J94," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B94" s="16"/>
       <x:c r="C94" s="16"/>
@@ -2937,7 +2937,7 @@
     </x:row>
     <x:row r="95" ht="15" hidden="0" customHeight="1">
       <x:c r="A95" s="16" t="str">
-        <x:f>IF(AND(B95="",C95=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B95&amp;C95," ",""))&amp;IF(E95&lt;&gt;"","-"&amp;RIGHT(E95,4),IF(J95&lt;&gt;"","-"&amp;RIGHT(J95,4),"")))</x:f>
+        <x:f>IF(AND(B95="",C95=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B95&amp;C95," ",""))&amp;IF(E95&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E95," ",""),4),IF(J95&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J95," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B95" s="16"/>
       <x:c r="C95" s="16"/>
@@ -2963,7 +2963,7 @@
     </x:row>
     <x:row r="96" ht="15" hidden="0" customHeight="1">
       <x:c r="A96" s="16" t="str">
-        <x:f>IF(AND(B96="",C96=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B96&amp;C96," ",""))&amp;IF(E96&lt;&gt;"","-"&amp;RIGHT(E96,4),IF(J96&lt;&gt;"","-"&amp;RIGHT(J96,4),"")))</x:f>
+        <x:f>IF(AND(B96="",C96=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B96&amp;C96," ",""))&amp;IF(E96&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E96," ",""),4),IF(J96&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J96," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B96" s="16"/>
       <x:c r="C96" s="16"/>
@@ -2989,7 +2989,7 @@
     </x:row>
     <x:row r="97" ht="15" hidden="0" customHeight="1">
       <x:c r="A97" s="16" t="str">
-        <x:f>IF(AND(B97="",C97=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B97&amp;C97," ",""))&amp;IF(E97&lt;&gt;"","-"&amp;RIGHT(E97,4),IF(J97&lt;&gt;"","-"&amp;RIGHT(J97,4),"")))</x:f>
+        <x:f>IF(AND(B97="",C97=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B97&amp;C97," ",""))&amp;IF(E97&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E97," ",""),4),IF(J97&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J97," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B97" s="16"/>
       <x:c r="C97" s="16"/>
@@ -3015,7 +3015,7 @@
     </x:row>
     <x:row r="98" ht="15" hidden="0" customHeight="1">
       <x:c r="A98" s="16" t="str">
-        <x:f>IF(AND(B98="",C98=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B98&amp;C98," ",""))&amp;IF(E98&lt;&gt;"","-"&amp;RIGHT(E98,4),IF(J98&lt;&gt;"","-"&amp;RIGHT(J98,4),"")))</x:f>
+        <x:f>IF(AND(B98="",C98=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B98&amp;C98," ",""))&amp;IF(E98&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E98," ",""),4),IF(J98&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J98," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B98" s="16"/>
       <x:c r="C98" s="16"/>
@@ -3041,7 +3041,7 @@
     </x:row>
     <x:row r="99" ht="15" hidden="0" customHeight="1">
       <x:c r="A99" s="16" t="str">
-        <x:f>IF(AND(B99="",C99=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B99&amp;C99," ",""))&amp;IF(E99&lt;&gt;"","-"&amp;RIGHT(E99,4),IF(J99&lt;&gt;"","-"&amp;RIGHT(J99,4),"")))</x:f>
+        <x:f>IF(AND(B99="",C99=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B99&amp;C99," ",""))&amp;IF(E99&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E99," ",""),4),IF(J99&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J99," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B99" s="16"/>
       <x:c r="C99" s="16"/>
@@ -3067,7 +3067,7 @@
     </x:row>
     <x:row r="100" ht="15" hidden="0" customHeight="1">
       <x:c r="A100" s="16" t="str">
-        <x:f>IF(AND(B100="",C100=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B100&amp;C100," ",""))&amp;IF(E100&lt;&gt;"","-"&amp;RIGHT(E100,4),IF(J100&lt;&gt;"","-"&amp;RIGHT(J100,4),"")))</x:f>
+        <x:f>IF(AND(B100="",C100=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B100&amp;C100," ",""))&amp;IF(E100&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E100," ",""),4),IF(J100&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J100," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B100" s="16"/>
       <x:c r="C100" s="16"/>
@@ -3093,7 +3093,7 @@
     </x:row>
     <x:row r="101" ht="15" hidden="0" customHeight="1">
       <x:c r="A101" s="16" t="str">
-        <x:f>IF(AND(B101="",C101=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B101&amp;C101," ",""))&amp;IF(E101&lt;&gt;"","-"&amp;RIGHT(E101,4),IF(J101&lt;&gt;"","-"&amp;RIGHT(J101,4),"")))</x:f>
+        <x:f>IF(AND(B101="",C101=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B101&amp;C101," ",""))&amp;IF(E101&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E101," ",""),4),IF(J101&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J101," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B101" s="16"/>
       <x:c r="C101" s="16"/>
@@ -3119,7 +3119,7 @@
     </x:row>
     <x:row r="102" ht="15" hidden="0" customHeight="1">
       <x:c r="A102" s="16" t="str">
-        <x:f>IF(AND(B102="",C102=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B102&amp;C102," ",""))&amp;IF(E102&lt;&gt;"","-"&amp;RIGHT(E102,4),IF(J102&lt;&gt;"","-"&amp;RIGHT(J102,4),"")))</x:f>
+        <x:f>IF(AND(B102="",C102=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B102&amp;C102," ",""))&amp;IF(E102&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E102," ",""),4),IF(J102&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J102," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B102" s="16"/>
       <x:c r="C102" s="16"/>
@@ -3145,7 +3145,7 @@
     </x:row>
     <x:row r="103" ht="15" hidden="0" customHeight="1">
       <x:c r="A103" s="16" t="str">
-        <x:f>IF(AND(B103="",C103=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B103&amp;C103," ",""))&amp;IF(E103&lt;&gt;"","-"&amp;RIGHT(E103,4),IF(J103&lt;&gt;"","-"&amp;RIGHT(J103,4),"")))</x:f>
+        <x:f>IF(AND(B103="",C103=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B103&amp;C103," ",""))&amp;IF(E103&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E103," ",""),4),IF(J103&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J103," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B103" s="16"/>
       <x:c r="C103" s="16"/>
@@ -3171,7 +3171,7 @@
     </x:row>
     <x:row r="104" ht="15" hidden="0" customHeight="1">
       <x:c r="A104" s="16" t="str">
-        <x:f>IF(AND(B104="",C104=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B104&amp;C104," ",""))&amp;IF(E104&lt;&gt;"","-"&amp;RIGHT(E104,4),IF(J104&lt;&gt;"","-"&amp;RIGHT(J104,4),"")))</x:f>
+        <x:f>IF(AND(B104="",C104=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B104&amp;C104," ",""))&amp;IF(E104&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E104," ",""),4),IF(J104&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J104," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B104" s="16"/>
       <x:c r="C104" s="16"/>
@@ -3197,7 +3197,7 @@
     </x:row>
     <x:row r="105" ht="15" hidden="0" customHeight="1">
       <x:c r="A105" s="16" t="str">
-        <x:f>IF(AND(B105="",C105=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B105&amp;C105," ",""))&amp;IF(E105&lt;&gt;"","-"&amp;RIGHT(E105,4),IF(J105&lt;&gt;"","-"&amp;RIGHT(J105,4),"")))</x:f>
+        <x:f>IF(AND(B105="",C105=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B105&amp;C105," ",""))&amp;IF(E105&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E105," ",""),4),IF(J105&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J105," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B105" s="16"/>
       <x:c r="C105" s="16"/>
@@ -3223,7 +3223,7 @@
     </x:row>
     <x:row r="106" ht="15" hidden="0" customHeight="1">
       <x:c r="A106" s="16" t="str">
-        <x:f>IF(AND(B106="",C106=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B106&amp;C106," ",""))&amp;IF(E106&lt;&gt;"","-"&amp;RIGHT(E106,4),IF(J106&lt;&gt;"","-"&amp;RIGHT(J106,4),"")))</x:f>
+        <x:f>IF(AND(B106="",C106=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B106&amp;C106," ",""))&amp;IF(E106&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E106," ",""),4),IF(J106&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J106," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B106" s="16"/>
       <x:c r="C106" s="16"/>
@@ -3249,7 +3249,7 @@
     </x:row>
     <x:row r="107" ht="15" hidden="0" customHeight="1">
       <x:c r="A107" s="16" t="str">
-        <x:f>IF(AND(B107="",C107=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B107&amp;C107," ",""))&amp;IF(E107&lt;&gt;"","-"&amp;RIGHT(E107,4),IF(J107&lt;&gt;"","-"&amp;RIGHT(J107,4),"")))</x:f>
+        <x:f>IF(AND(B107="",C107=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B107&amp;C107," ",""))&amp;IF(E107&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E107," ",""),4),IF(J107&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J107," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B107" s="16"/>
       <x:c r="C107" s="16"/>
@@ -3275,7 +3275,7 @@
     </x:row>
     <x:row r="108" ht="15" hidden="0" customHeight="1">
       <x:c r="A108" s="16" t="str">
-        <x:f>IF(AND(B108="",C108=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B108&amp;C108," ",""))&amp;IF(E108&lt;&gt;"","-"&amp;RIGHT(E108,4),IF(J108&lt;&gt;"","-"&amp;RIGHT(J108,4),"")))</x:f>
+        <x:f>IF(AND(B108="",C108=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B108&amp;C108," ",""))&amp;IF(E108&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E108," ",""),4),IF(J108&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J108," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B108" s="16"/>
       <x:c r="C108" s="16"/>
@@ -3301,7 +3301,7 @@
     </x:row>
     <x:row r="109" ht="15" hidden="0" customHeight="1">
       <x:c r="A109" s="16" t="str">
-        <x:f>IF(AND(B109="",C109=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B109&amp;C109," ",""))&amp;IF(E109&lt;&gt;"","-"&amp;RIGHT(E109,4),IF(J109&lt;&gt;"","-"&amp;RIGHT(J109,4),"")))</x:f>
+        <x:f>IF(AND(B109="",C109=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B109&amp;C109," ",""))&amp;IF(E109&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E109," ",""),4),IF(J109&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J109," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B109" s="16"/>
       <x:c r="C109" s="16"/>
@@ -3327,7 +3327,7 @@
     </x:row>
     <x:row r="110" ht="15" hidden="0" customHeight="1">
       <x:c r="A110" s="16" t="str">
-        <x:f>IF(AND(B110="",C110=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B110&amp;C110," ",""))&amp;IF(E110&lt;&gt;"","-"&amp;RIGHT(E110,4),IF(J110&lt;&gt;"","-"&amp;RIGHT(J110,4),"")))</x:f>
+        <x:f>IF(AND(B110="",C110=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B110&amp;C110," ",""))&amp;IF(E110&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E110," ",""),4),IF(J110&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J110," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B110" s="16"/>
       <x:c r="C110" s="16"/>
@@ -3353,7 +3353,7 @@
     </x:row>
     <x:row r="111" ht="15" hidden="0" customHeight="1">
       <x:c r="A111" s="16" t="str">
-        <x:f>IF(AND(B111="",C111=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B111&amp;C111," ",""))&amp;IF(E111&lt;&gt;"","-"&amp;RIGHT(E111,4),IF(J111&lt;&gt;"","-"&amp;RIGHT(J111,4),"")))</x:f>
+        <x:f>IF(AND(B111="",C111=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B111&amp;C111," ",""))&amp;IF(E111&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E111," ",""),4),IF(J111&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J111," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B111" s="16"/>
       <x:c r="C111" s="16"/>
@@ -3379,7 +3379,7 @@
     </x:row>
     <x:row r="112" ht="15" hidden="0" customHeight="1">
       <x:c r="A112" s="16" t="str">
-        <x:f>IF(AND(B112="",C112=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B112&amp;C112," ",""))&amp;IF(E112&lt;&gt;"","-"&amp;RIGHT(E112,4),IF(J112&lt;&gt;"","-"&amp;RIGHT(J112,4),"")))</x:f>
+        <x:f>IF(AND(B112="",C112=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B112&amp;C112," ",""))&amp;IF(E112&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E112," ",""),4),IF(J112&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J112," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B112" s="16"/>
       <x:c r="C112" s="16"/>
@@ -3405,7 +3405,7 @@
     </x:row>
     <x:row r="113" ht="15" hidden="0" customHeight="1">
       <x:c r="A113" s="16" t="str">
-        <x:f>IF(AND(B113="",C113=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B113&amp;C113," ",""))&amp;IF(E113&lt;&gt;"","-"&amp;RIGHT(E113,4),IF(J113&lt;&gt;"","-"&amp;RIGHT(J113,4),"")))</x:f>
+        <x:f>IF(AND(B113="",C113=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B113&amp;C113," ",""))&amp;IF(E113&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E113," ",""),4),IF(J113&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J113," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B113" s="16"/>
       <x:c r="C113" s="16"/>
@@ -3431,7 +3431,7 @@
     </x:row>
     <x:row r="114" ht="15" hidden="0" customHeight="1">
       <x:c r="A114" s="16" t="str">
-        <x:f>IF(AND(B114="",C114=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B114&amp;C114," ",""))&amp;IF(E114&lt;&gt;"","-"&amp;RIGHT(E114,4),IF(J114&lt;&gt;"","-"&amp;RIGHT(J114,4),"")))</x:f>
+        <x:f>IF(AND(B114="",C114=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B114&amp;C114," ",""))&amp;IF(E114&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E114," ",""),4),IF(J114&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J114," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B114" s="16"/>
       <x:c r="C114" s="16"/>
@@ -3457,7 +3457,7 @@
     </x:row>
     <x:row r="115" ht="15" hidden="0" customHeight="1">
       <x:c r="A115" s="16" t="str">
-        <x:f>IF(AND(B115="",C115=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B115&amp;C115," ",""))&amp;IF(E115&lt;&gt;"","-"&amp;RIGHT(E115,4),IF(J115&lt;&gt;"","-"&amp;RIGHT(J115,4),"")))</x:f>
+        <x:f>IF(AND(B115="",C115=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B115&amp;C115," ",""))&amp;IF(E115&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E115," ",""),4),IF(J115&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J115," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B115" s="16"/>
       <x:c r="C115" s="16"/>
@@ -3483,7 +3483,7 @@
     </x:row>
     <x:row r="116" ht="15" hidden="0" customHeight="1">
       <x:c r="A116" s="16" t="str">
-        <x:f>IF(AND(B116="",C116=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B116&amp;C116," ",""))&amp;IF(E116&lt;&gt;"","-"&amp;RIGHT(E116,4),IF(J116&lt;&gt;"","-"&amp;RIGHT(J116,4),"")))</x:f>
+        <x:f>IF(AND(B116="",C116=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B116&amp;C116," ",""))&amp;IF(E116&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E116," ",""),4),IF(J116&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J116," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B116" s="16"/>
       <x:c r="C116" s="16"/>
@@ -3509,7 +3509,7 @@
     </x:row>
     <x:row r="117" ht="15" hidden="0" customHeight="1">
       <x:c r="A117" s="16" t="str">
-        <x:f>IF(AND(B117="",C117=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B117&amp;C117," ",""))&amp;IF(E117&lt;&gt;"","-"&amp;RIGHT(E117,4),IF(J117&lt;&gt;"","-"&amp;RIGHT(J117,4),"")))</x:f>
+        <x:f>IF(AND(B117="",C117=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B117&amp;C117," ",""))&amp;IF(E117&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E117," ",""),4),IF(J117&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J117," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B117" s="16"/>
       <x:c r="C117" s="16"/>
@@ -3535,7 +3535,7 @@
     </x:row>
     <x:row r="118" ht="15" hidden="0" customHeight="1">
       <x:c r="A118" s="16" t="str">
-        <x:f>IF(AND(B118="",C118=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B118&amp;C118," ",""))&amp;IF(E118&lt;&gt;"","-"&amp;RIGHT(E118,4),IF(J118&lt;&gt;"","-"&amp;RIGHT(J118,4),"")))</x:f>
+        <x:f>IF(AND(B118="",C118=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B118&amp;C118," ",""))&amp;IF(E118&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E118," ",""),4),IF(J118&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J118," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B118" s="16"/>
       <x:c r="C118" s="16"/>
@@ -3561,7 +3561,7 @@
     </x:row>
     <x:row r="119" ht="15" hidden="0" customHeight="1">
       <x:c r="A119" s="16" t="str">
-        <x:f>IF(AND(B119="",C119=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B119&amp;C119," ",""))&amp;IF(E119&lt;&gt;"","-"&amp;RIGHT(E119,4),IF(J119&lt;&gt;"","-"&amp;RIGHT(J119,4),"")))</x:f>
+        <x:f>IF(AND(B119="",C119=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B119&amp;C119," ",""))&amp;IF(E119&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E119," ",""),4),IF(J119&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J119," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B119" s="16"/>
       <x:c r="C119" s="16"/>
@@ -3587,7 +3587,7 @@
     </x:row>
     <x:row r="120" ht="15" hidden="0" customHeight="1">
       <x:c r="A120" s="16" t="str">
-        <x:f>IF(AND(B120="",C120=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B120&amp;C120," ",""))&amp;IF(E120&lt;&gt;"","-"&amp;RIGHT(E120,4),IF(J120&lt;&gt;"","-"&amp;RIGHT(J120,4),"")))</x:f>
+        <x:f>IF(AND(B120="",C120=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B120&amp;C120," ",""))&amp;IF(E120&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E120," ",""),4),IF(J120&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J120," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B120" s="16"/>
       <x:c r="C120" s="16"/>
@@ -3613,7 +3613,7 @@
     </x:row>
     <x:row r="121" ht="15" hidden="0" customHeight="1">
       <x:c r="A121" s="16" t="str">
-        <x:f>IF(AND(B121="",C121=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B121&amp;C121," ",""))&amp;IF(E121&lt;&gt;"","-"&amp;RIGHT(E121,4),IF(J121&lt;&gt;"","-"&amp;RIGHT(J121,4),"")))</x:f>
+        <x:f>IF(AND(B121="",C121=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B121&amp;C121," ",""))&amp;IF(E121&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E121," ",""),4),IF(J121&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J121," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B121" s="16"/>
       <x:c r="C121" s="16"/>
@@ -3639,7 +3639,7 @@
     </x:row>
     <x:row r="122" ht="15" hidden="0" customHeight="1">
       <x:c r="A122" s="16" t="str">
-        <x:f>IF(AND(B122="",C122=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B122&amp;C122," ",""))&amp;IF(E122&lt;&gt;"","-"&amp;RIGHT(E122,4),IF(J122&lt;&gt;"","-"&amp;RIGHT(J122,4),"")))</x:f>
+        <x:f>IF(AND(B122="",C122=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B122&amp;C122," ",""))&amp;IF(E122&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E122," ",""),4),IF(J122&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J122," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B122" s="16"/>
       <x:c r="C122" s="16"/>
@@ -3665,7 +3665,7 @@
     </x:row>
     <x:row r="123" ht="15" hidden="0" customHeight="1">
       <x:c r="A123" s="16" t="str">
-        <x:f>IF(AND(B123="",C123=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B123&amp;C123," ",""))&amp;IF(E123&lt;&gt;"","-"&amp;RIGHT(E123,4),IF(J123&lt;&gt;"","-"&amp;RIGHT(J123,4),"")))</x:f>
+        <x:f>IF(AND(B123="",C123=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B123&amp;C123," ",""))&amp;IF(E123&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E123," ",""),4),IF(J123&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J123," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B123" s="16"/>
       <x:c r="C123" s="16"/>
@@ -3691,7 +3691,7 @@
     </x:row>
     <x:row r="124" ht="15" hidden="0" customHeight="1">
       <x:c r="A124" s="16" t="str">
-        <x:f>IF(AND(B124="",C124=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B124&amp;C124," ",""))&amp;IF(E124&lt;&gt;"","-"&amp;RIGHT(E124,4),IF(J124&lt;&gt;"","-"&amp;RIGHT(J124,4),"")))</x:f>
+        <x:f>IF(AND(B124="",C124=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B124&amp;C124," ",""))&amp;IF(E124&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E124," ",""),4),IF(J124&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J124," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B124" s="16"/>
       <x:c r="C124" s="16"/>
@@ -3717,7 +3717,7 @@
     </x:row>
     <x:row r="125" ht="15" hidden="0" customHeight="1">
       <x:c r="A125" s="16" t="str">
-        <x:f>IF(AND(B125="",C125=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B125&amp;C125," ",""))&amp;IF(E125&lt;&gt;"","-"&amp;RIGHT(E125,4),IF(J125&lt;&gt;"","-"&amp;RIGHT(J125,4),"")))</x:f>
+        <x:f>IF(AND(B125="",C125=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B125&amp;C125," ",""))&amp;IF(E125&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E125," ",""),4),IF(J125&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J125," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B125" s="16"/>
       <x:c r="C125" s="16"/>
@@ -3743,7 +3743,7 @@
     </x:row>
     <x:row r="126" ht="15" hidden="0" customHeight="1">
       <x:c r="A126" s="16" t="str">
-        <x:f>IF(AND(B126="",C126=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B126&amp;C126," ",""))&amp;IF(E126&lt;&gt;"","-"&amp;RIGHT(E126,4),IF(J126&lt;&gt;"","-"&amp;RIGHT(J126,4),"")))</x:f>
+        <x:f>IF(AND(B126="",C126=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B126&amp;C126," ",""))&amp;IF(E126&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E126," ",""),4),IF(J126&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J126," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B126" s="16"/>
       <x:c r="C126" s="16"/>
@@ -3769,7 +3769,7 @@
     </x:row>
     <x:row r="127" ht="15" hidden="0" customHeight="1">
       <x:c r="A127" s="16" t="str">
-        <x:f>IF(AND(B127="",C127=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B127&amp;C127," ",""))&amp;IF(E127&lt;&gt;"","-"&amp;RIGHT(E127,4),IF(J127&lt;&gt;"","-"&amp;RIGHT(J127,4),"")))</x:f>
+        <x:f>IF(AND(B127="",C127=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B127&amp;C127," ",""))&amp;IF(E127&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E127," ",""),4),IF(J127&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J127," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B127" s="16"/>
       <x:c r="C127" s="16"/>
@@ -3795,7 +3795,7 @@
     </x:row>
     <x:row r="128" ht="15" hidden="0" customHeight="1">
       <x:c r="A128" s="16" t="str">
-        <x:f>IF(AND(B128="",C128=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B128&amp;C128," ",""))&amp;IF(E128&lt;&gt;"","-"&amp;RIGHT(E128,4),IF(J128&lt;&gt;"","-"&amp;RIGHT(J128,4),"")))</x:f>
+        <x:f>IF(AND(B128="",C128=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B128&amp;C128," ",""))&amp;IF(E128&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E128," ",""),4),IF(J128&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J128," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B128" s="16"/>
       <x:c r="C128" s="16"/>
@@ -3821,7 +3821,7 @@
     </x:row>
     <x:row r="129" ht="15" hidden="0" customHeight="1">
       <x:c r="A129" s="16" t="str">
-        <x:f>IF(AND(B129="",C129=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B129&amp;C129," ",""))&amp;IF(E129&lt;&gt;"","-"&amp;RIGHT(E129,4),IF(J129&lt;&gt;"","-"&amp;RIGHT(J129,4),"")))</x:f>
+        <x:f>IF(AND(B129="",C129=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B129&amp;C129," ",""))&amp;IF(E129&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E129," ",""),4),IF(J129&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J129," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B129" s="16"/>
       <x:c r="C129" s="16"/>
@@ -3847,7 +3847,7 @@
     </x:row>
     <x:row r="130" ht="15" hidden="0" customHeight="1">
       <x:c r="A130" s="16" t="str">
-        <x:f>IF(AND(B130="",C130=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B130&amp;C130," ",""))&amp;IF(E130&lt;&gt;"","-"&amp;RIGHT(E130,4),IF(J130&lt;&gt;"","-"&amp;RIGHT(J130,4),"")))</x:f>
+        <x:f>IF(AND(B130="",C130=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B130&amp;C130," ",""))&amp;IF(E130&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E130," ",""),4),IF(J130&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J130," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B130" s="16"/>
       <x:c r="C130" s="16"/>
@@ -3873,7 +3873,7 @@
     </x:row>
     <x:row r="131" ht="15" hidden="0" customHeight="1">
       <x:c r="A131" s="16" t="str">
-        <x:f>IF(AND(B131="",C131=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B131&amp;C131," ",""))&amp;IF(E131&lt;&gt;"","-"&amp;RIGHT(E131,4),IF(J131&lt;&gt;"","-"&amp;RIGHT(J131,4),"")))</x:f>
+        <x:f>IF(AND(B131="",C131=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B131&amp;C131," ",""))&amp;IF(E131&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E131," ",""),4),IF(J131&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J131," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B131" s="16"/>
       <x:c r="C131" s="16"/>
@@ -3899,7 +3899,7 @@
     </x:row>
     <x:row r="132" ht="15" hidden="0" customHeight="1">
       <x:c r="A132" s="16" t="str">
-        <x:f>IF(AND(B132="",C132=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B132&amp;C132," ",""))&amp;IF(E132&lt;&gt;"","-"&amp;RIGHT(E132,4),IF(J132&lt;&gt;"","-"&amp;RIGHT(J132,4),"")))</x:f>
+        <x:f>IF(AND(B132="",C132=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B132&amp;C132," ",""))&amp;IF(E132&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E132," ",""),4),IF(J132&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J132," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B132" s="16"/>
       <x:c r="C132" s="16"/>
@@ -3925,7 +3925,7 @@
     </x:row>
     <x:row r="133" ht="15" hidden="0" customHeight="1">
       <x:c r="A133" s="16" t="str">
-        <x:f>IF(AND(B133="",C133=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B133&amp;C133," ",""))&amp;IF(E133&lt;&gt;"","-"&amp;RIGHT(E133,4),IF(J133&lt;&gt;"","-"&amp;RIGHT(J133,4),"")))</x:f>
+        <x:f>IF(AND(B133="",C133=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B133&amp;C133," ",""))&amp;IF(E133&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E133," ",""),4),IF(J133&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J133," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B133" s="16"/>
       <x:c r="C133" s="16"/>
@@ -3951,7 +3951,7 @@
     </x:row>
     <x:row r="134" ht="15" hidden="0" customHeight="1">
       <x:c r="A134" s="16" t="str">
-        <x:f>IF(AND(B134="",C134=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B134&amp;C134," ",""))&amp;IF(E134&lt;&gt;"","-"&amp;RIGHT(E134,4),IF(J134&lt;&gt;"","-"&amp;RIGHT(J134,4),"")))</x:f>
+        <x:f>IF(AND(B134="",C134=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B134&amp;C134," ",""))&amp;IF(E134&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E134," ",""),4),IF(J134&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J134," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B134" s="16"/>
       <x:c r="C134" s="16"/>
@@ -3977,7 +3977,7 @@
     </x:row>
     <x:row r="135" ht="15" hidden="0" customHeight="1">
       <x:c r="A135" s="16" t="str">
-        <x:f>IF(AND(B135="",C135=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B135&amp;C135," ",""))&amp;IF(E135&lt;&gt;"","-"&amp;RIGHT(E135,4),IF(J135&lt;&gt;"","-"&amp;RIGHT(J135,4),"")))</x:f>
+        <x:f>IF(AND(B135="",C135=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B135&amp;C135," ",""))&amp;IF(E135&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E135," ",""),4),IF(J135&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J135," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B135" s="16"/>
       <x:c r="C135" s="16"/>
@@ -4003,7 +4003,7 @@
     </x:row>
     <x:row r="136" ht="15" hidden="0" customHeight="1">
       <x:c r="A136" s="16" t="str">
-        <x:f>IF(AND(B136="",C136=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B136&amp;C136," ",""))&amp;IF(E136&lt;&gt;"","-"&amp;RIGHT(E136,4),IF(J136&lt;&gt;"","-"&amp;RIGHT(J136,4),"")))</x:f>
+        <x:f>IF(AND(B136="",C136=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B136&amp;C136," ",""))&amp;IF(E136&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E136," ",""),4),IF(J136&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J136," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B136" s="16"/>
       <x:c r="C136" s="16"/>
@@ -4029,7 +4029,7 @@
     </x:row>
     <x:row r="137" ht="15" hidden="0" customHeight="1">
       <x:c r="A137" s="16" t="str">
-        <x:f>IF(AND(B137="",C137=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B137&amp;C137," ",""))&amp;IF(E137&lt;&gt;"","-"&amp;RIGHT(E137,4),IF(J137&lt;&gt;"","-"&amp;RIGHT(J137,4),"")))</x:f>
+        <x:f>IF(AND(B137="",C137=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B137&amp;C137," ",""))&amp;IF(E137&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E137," ",""),4),IF(J137&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J137," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B137" s="16"/>
       <x:c r="C137" s="16"/>
@@ -4055,7 +4055,7 @@
     </x:row>
     <x:row r="138" ht="15" hidden="0" customHeight="1">
       <x:c r="A138" s="16" t="str">
-        <x:f>IF(AND(B138="",C138=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B138&amp;C138," ",""))&amp;IF(E138&lt;&gt;"","-"&amp;RIGHT(E138,4),IF(J138&lt;&gt;"","-"&amp;RIGHT(J138,4),"")))</x:f>
+        <x:f>IF(AND(B138="",C138=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B138&amp;C138," ",""))&amp;IF(E138&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E138," ",""),4),IF(J138&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J138," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B138" s="16"/>
       <x:c r="C138" s="16"/>
@@ -4081,7 +4081,7 @@
     </x:row>
     <x:row r="139" ht="15" hidden="0" customHeight="1">
       <x:c r="A139" s="16" t="str">
-        <x:f>IF(AND(B139="",C139=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B139&amp;C139," ",""))&amp;IF(E139&lt;&gt;"","-"&amp;RIGHT(E139,4),IF(J139&lt;&gt;"","-"&amp;RIGHT(J139,4),"")))</x:f>
+        <x:f>IF(AND(B139="",C139=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B139&amp;C139," ",""))&amp;IF(E139&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E139," ",""),4),IF(J139&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J139," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B139" s="16"/>
       <x:c r="C139" s="16"/>
@@ -4107,7 +4107,7 @@
     </x:row>
     <x:row r="140" ht="15" hidden="0" customHeight="1">
       <x:c r="A140" s="16" t="str">
-        <x:f>IF(AND(B140="",C140=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B140&amp;C140," ",""))&amp;IF(E140&lt;&gt;"","-"&amp;RIGHT(E140,4),IF(J140&lt;&gt;"","-"&amp;RIGHT(J140,4),"")))</x:f>
+        <x:f>IF(AND(B140="",C140=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B140&amp;C140," ",""))&amp;IF(E140&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E140," ",""),4),IF(J140&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J140," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B140" s="16"/>
       <x:c r="C140" s="16"/>
@@ -4133,7 +4133,7 @@
     </x:row>
     <x:row r="141" ht="15" hidden="0" customHeight="1">
       <x:c r="A141" s="16" t="str">
-        <x:f>IF(AND(B141="",C141=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B141&amp;C141," ",""))&amp;IF(E141&lt;&gt;"","-"&amp;RIGHT(E141,4),IF(J141&lt;&gt;"","-"&amp;RIGHT(J141,4),"")))</x:f>
+        <x:f>IF(AND(B141="",C141=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B141&amp;C141," ",""))&amp;IF(E141&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E141," ",""),4),IF(J141&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J141," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B141" s="16"/>
       <x:c r="C141" s="16"/>
@@ -4159,7 +4159,7 @@
     </x:row>
     <x:row r="142" ht="15" hidden="0" customHeight="1">
       <x:c r="A142" s="16" t="str">
-        <x:f>IF(AND(B142="",C142=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B142&amp;C142," ",""))&amp;IF(E142&lt;&gt;"","-"&amp;RIGHT(E142,4),IF(J142&lt;&gt;"","-"&amp;RIGHT(J142,4),"")))</x:f>
+        <x:f>IF(AND(B142="",C142=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B142&amp;C142," ",""))&amp;IF(E142&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E142," ",""),4),IF(J142&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J142," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B142" s="16"/>
       <x:c r="C142" s="16"/>
@@ -4185,7 +4185,7 @@
     </x:row>
     <x:row r="143" ht="15" hidden="0" customHeight="1">
       <x:c r="A143" s="16" t="str">
-        <x:f>IF(AND(B143="",C143=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B143&amp;C143," ",""))&amp;IF(E143&lt;&gt;"","-"&amp;RIGHT(E143,4),IF(J143&lt;&gt;"","-"&amp;RIGHT(J143,4),"")))</x:f>
+        <x:f>IF(AND(B143="",C143=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B143&amp;C143," ",""))&amp;IF(E143&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E143," ",""),4),IF(J143&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J143," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B143" s="16"/>
       <x:c r="C143" s="16"/>
@@ -4211,7 +4211,7 @@
     </x:row>
     <x:row r="144" ht="15" hidden="0" customHeight="1">
       <x:c r="A144" s="16" t="str">
-        <x:f>IF(AND(B144="",C144=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B144&amp;C144," ",""))&amp;IF(E144&lt;&gt;"","-"&amp;RIGHT(E144,4),IF(J144&lt;&gt;"","-"&amp;RIGHT(J144,4),"")))</x:f>
+        <x:f>IF(AND(B144="",C144=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B144&amp;C144," ",""))&amp;IF(E144&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E144," ",""),4),IF(J144&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J144," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B144" s="16"/>
       <x:c r="C144" s="16"/>
@@ -4237,7 +4237,7 @@
     </x:row>
     <x:row r="145" ht="15" hidden="0" customHeight="1">
       <x:c r="A145" s="16" t="str">
-        <x:f>IF(AND(B145="",C145=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B145&amp;C145," ",""))&amp;IF(E145&lt;&gt;"","-"&amp;RIGHT(E145,4),IF(J145&lt;&gt;"","-"&amp;RIGHT(J145,4),"")))</x:f>
+        <x:f>IF(AND(B145="",C145=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B145&amp;C145," ",""))&amp;IF(E145&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E145," ",""),4),IF(J145&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J145," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B145" s="16"/>
       <x:c r="C145" s="16"/>
@@ -4263,7 +4263,7 @@
     </x:row>
     <x:row r="146" ht="15" hidden="0" customHeight="1">
       <x:c r="A146" s="16" t="str">
-        <x:f>IF(AND(B146="",C146=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B146&amp;C146," ",""))&amp;IF(E146&lt;&gt;"","-"&amp;RIGHT(E146,4),IF(J146&lt;&gt;"","-"&amp;RIGHT(J146,4),"")))</x:f>
+        <x:f>IF(AND(B146="",C146=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B146&amp;C146," ",""))&amp;IF(E146&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E146," ",""),4),IF(J146&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J146," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B146" s="16"/>
       <x:c r="C146" s="16"/>
@@ -4289,7 +4289,7 @@
     </x:row>
     <x:row r="147" ht="15" hidden="0" customHeight="1">
       <x:c r="A147" s="16" t="str">
-        <x:f>IF(AND(B147="",C147=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B147&amp;C147," ",""))&amp;IF(E147&lt;&gt;"","-"&amp;RIGHT(E147,4),IF(J147&lt;&gt;"","-"&amp;RIGHT(J147,4),"")))</x:f>
+        <x:f>IF(AND(B147="",C147=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B147&amp;C147," ",""))&amp;IF(E147&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E147," ",""),4),IF(J147&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J147," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B147" s="16"/>
       <x:c r="C147" s="16"/>
@@ -4315,7 +4315,7 @@
     </x:row>
     <x:row r="148" ht="15" hidden="0" customHeight="1">
       <x:c r="A148" s="16" t="str">
-        <x:f>IF(AND(B148="",C148=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B148&amp;C148," ",""))&amp;IF(E148&lt;&gt;"","-"&amp;RIGHT(E148,4),IF(J148&lt;&gt;"","-"&amp;RIGHT(J148,4),"")))</x:f>
+        <x:f>IF(AND(B148="",C148=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B148&amp;C148," ",""))&amp;IF(E148&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E148," ",""),4),IF(J148&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J148," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B148" s="16"/>
       <x:c r="C148" s="16"/>
@@ -4341,7 +4341,7 @@
     </x:row>
     <x:row r="149" ht="15" hidden="0" customHeight="1">
       <x:c r="A149" s="16" t="str">
-        <x:f>IF(AND(B149="",C149=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B149&amp;C149," ",""))&amp;IF(E149&lt;&gt;"","-"&amp;RIGHT(E149,4),IF(J149&lt;&gt;"","-"&amp;RIGHT(J149,4),"")))</x:f>
+        <x:f>IF(AND(B149="",C149=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B149&amp;C149," ",""))&amp;IF(E149&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E149," ",""),4),IF(J149&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J149," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B149" s="16"/>
       <x:c r="C149" s="16"/>
@@ -4367,7 +4367,7 @@
     </x:row>
     <x:row r="150" ht="15" hidden="0" customHeight="1">
       <x:c r="A150" s="16" t="str">
-        <x:f>IF(AND(B150="",C150=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B150&amp;C150," ",""))&amp;IF(E150&lt;&gt;"","-"&amp;RIGHT(E150,4),IF(J150&lt;&gt;"","-"&amp;RIGHT(J150,4),"")))</x:f>
+        <x:f>IF(AND(B150="",C150=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B150&amp;C150," ",""))&amp;IF(E150&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E150," ",""),4),IF(J150&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J150," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B150" s="16"/>
       <x:c r="C150" s="16"/>
@@ -4393,7 +4393,7 @@
     </x:row>
     <x:row r="151" ht="15" hidden="0" customHeight="1">
       <x:c r="A151" s="16" t="str">
-        <x:f>IF(AND(B151="",C151=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B151&amp;C151," ",""))&amp;IF(E151&lt;&gt;"","-"&amp;RIGHT(E151,4),IF(J151&lt;&gt;"","-"&amp;RIGHT(J151,4),"")))</x:f>
+        <x:f>IF(AND(B151="",C151=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B151&amp;C151," ",""))&amp;IF(E151&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E151," ",""),4),IF(J151&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J151," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B151" s="16"/>
       <x:c r="C151" s="16"/>
@@ -4419,7 +4419,7 @@
     </x:row>
     <x:row r="152" ht="15" hidden="0" customHeight="1">
       <x:c r="A152" s="16" t="str">
-        <x:f>IF(AND(B152="",C152=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B152&amp;C152," ",""))&amp;IF(E152&lt;&gt;"","-"&amp;RIGHT(E152,4),IF(J152&lt;&gt;"","-"&amp;RIGHT(J152,4),"")))</x:f>
+        <x:f>IF(AND(B152="",C152=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B152&amp;C152," ",""))&amp;IF(E152&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E152," ",""),4),IF(J152&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J152," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B152" s="16"/>
       <x:c r="C152" s="16"/>
@@ -4445,7 +4445,7 @@
     </x:row>
     <x:row r="153" ht="15" hidden="0" customHeight="1">
       <x:c r="A153" s="16" t="str">
-        <x:f>IF(AND(B153="",C153=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B153&amp;C153," ",""))&amp;IF(E153&lt;&gt;"","-"&amp;RIGHT(E153,4),IF(J153&lt;&gt;"","-"&amp;RIGHT(J153,4),"")))</x:f>
+        <x:f>IF(AND(B153="",C153=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B153&amp;C153," ",""))&amp;IF(E153&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E153," ",""),4),IF(J153&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J153," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B153" s="16"/>
       <x:c r="C153" s="16"/>
@@ -4471,7 +4471,7 @@
     </x:row>
     <x:row r="154" ht="15" hidden="0" customHeight="1">
       <x:c r="A154" s="16" t="str">
-        <x:f>IF(AND(B154="",C154=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B154&amp;C154," ",""))&amp;IF(E154&lt;&gt;"","-"&amp;RIGHT(E154,4),IF(J154&lt;&gt;"","-"&amp;RIGHT(J154,4),"")))</x:f>
+        <x:f>IF(AND(B154="",C154=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B154&amp;C154," ",""))&amp;IF(E154&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E154," ",""),4),IF(J154&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J154," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B154" s="16"/>
       <x:c r="C154" s="16"/>
@@ -4497,7 +4497,7 @@
     </x:row>
     <x:row r="155" ht="15" hidden="0" customHeight="1">
       <x:c r="A155" s="16" t="str">
-        <x:f>IF(AND(B155="",C155=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B155&amp;C155," ",""))&amp;IF(E155&lt;&gt;"","-"&amp;RIGHT(E155,4),IF(J155&lt;&gt;"","-"&amp;RIGHT(J155,4),"")))</x:f>
+        <x:f>IF(AND(B155="",C155=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B155&amp;C155," ",""))&amp;IF(E155&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E155," ",""),4),IF(J155&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J155," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B155" s="16"/>
       <x:c r="C155" s="16"/>
@@ -4523,7 +4523,7 @@
     </x:row>
     <x:row r="156" ht="15" hidden="0" customHeight="1">
       <x:c r="A156" s="16" t="str">
-        <x:f>IF(AND(B156="",C156=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B156&amp;C156," ",""))&amp;IF(E156&lt;&gt;"","-"&amp;RIGHT(E156,4),IF(J156&lt;&gt;"","-"&amp;RIGHT(J156,4),"")))</x:f>
+        <x:f>IF(AND(B156="",C156=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B156&amp;C156," ",""))&amp;IF(E156&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E156," ",""),4),IF(J156&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J156," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B156" s="16"/>
       <x:c r="C156" s="16"/>
@@ -4549,7 +4549,7 @@
     </x:row>
     <x:row r="157" ht="15" hidden="0" customHeight="1">
       <x:c r="A157" s="16" t="str">
-        <x:f>IF(AND(B157="",C157=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B157&amp;C157," ",""))&amp;IF(E157&lt;&gt;"","-"&amp;RIGHT(E157,4),IF(J157&lt;&gt;"","-"&amp;RIGHT(J157,4),"")))</x:f>
+        <x:f>IF(AND(B157="",C157=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B157&amp;C157," ",""))&amp;IF(E157&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E157," ",""),4),IF(J157&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J157," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B157" s="16"/>
       <x:c r="C157" s="16"/>
@@ -4575,7 +4575,7 @@
     </x:row>
     <x:row r="158" ht="15" hidden="0" customHeight="1">
       <x:c r="A158" s="16" t="str">
-        <x:f>IF(AND(B158="",C158=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B158&amp;C158," ",""))&amp;IF(E158&lt;&gt;"","-"&amp;RIGHT(E158,4),IF(J158&lt;&gt;"","-"&amp;RIGHT(J158,4),"")))</x:f>
+        <x:f>IF(AND(B158="",C158=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B158&amp;C158," ",""))&amp;IF(E158&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E158," ",""),4),IF(J158&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J158," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B158" s="16"/>
       <x:c r="C158" s="16"/>
@@ -4601,7 +4601,7 @@
     </x:row>
     <x:row r="159" ht="15" hidden="0" customHeight="1">
       <x:c r="A159" s="16" t="str">
-        <x:f>IF(AND(B159="",C159=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B159&amp;C159," ",""))&amp;IF(E159&lt;&gt;"","-"&amp;RIGHT(E159,4),IF(J159&lt;&gt;"","-"&amp;RIGHT(J159,4),"")))</x:f>
+        <x:f>IF(AND(B159="",C159=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B159&amp;C159," ",""))&amp;IF(E159&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E159," ",""),4),IF(J159&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J159," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B159" s="16"/>
       <x:c r="C159" s="16"/>
@@ -4627,7 +4627,7 @@
     </x:row>
     <x:row r="160" ht="15" hidden="0" customHeight="1">
       <x:c r="A160" s="16" t="str">
-        <x:f>IF(AND(B160="",C160=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B160&amp;C160," ",""))&amp;IF(E160&lt;&gt;"","-"&amp;RIGHT(E160,4),IF(J160&lt;&gt;"","-"&amp;RIGHT(J160,4),"")))</x:f>
+        <x:f>IF(AND(B160="",C160=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B160&amp;C160," ",""))&amp;IF(E160&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E160," ",""),4),IF(J160&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J160," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B160" s="16"/>
       <x:c r="C160" s="16"/>
@@ -4653,7 +4653,7 @@
     </x:row>
     <x:row r="161" ht="15" hidden="0" customHeight="1">
       <x:c r="A161" s="16" t="str">
-        <x:f>IF(AND(B161="",C161=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B161&amp;C161," ",""))&amp;IF(E161&lt;&gt;"","-"&amp;RIGHT(E161,4),IF(J161&lt;&gt;"","-"&amp;RIGHT(J161,4),"")))</x:f>
+        <x:f>IF(AND(B161="",C161=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B161&amp;C161," ",""))&amp;IF(E161&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E161," ",""),4),IF(J161&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J161," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B161" s="16"/>
       <x:c r="C161" s="16"/>
@@ -4679,7 +4679,7 @@
     </x:row>
     <x:row r="162" ht="15" hidden="0" customHeight="1">
       <x:c r="A162" s="16" t="str">
-        <x:f>IF(AND(B162="",C162=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B162&amp;C162," ",""))&amp;IF(E162&lt;&gt;"","-"&amp;RIGHT(E162,4),IF(J162&lt;&gt;"","-"&amp;RIGHT(J162,4),"")))</x:f>
+        <x:f>IF(AND(B162="",C162=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B162&amp;C162," ",""))&amp;IF(E162&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E162," ",""),4),IF(J162&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J162," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B162" s="16"/>
       <x:c r="C162" s="16"/>
@@ -4705,7 +4705,7 @@
     </x:row>
     <x:row r="163" ht="15" hidden="0" customHeight="1">
       <x:c r="A163" s="16" t="str">
-        <x:f>IF(AND(B163="",C163=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B163&amp;C163," ",""))&amp;IF(E163&lt;&gt;"","-"&amp;RIGHT(E163,4),IF(J163&lt;&gt;"","-"&amp;RIGHT(J163,4),"")))</x:f>
+        <x:f>IF(AND(B163="",C163=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B163&amp;C163," ",""))&amp;IF(E163&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E163," ",""),4),IF(J163&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J163," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B163" s="16"/>
       <x:c r="C163" s="16"/>
@@ -4731,7 +4731,7 @@
     </x:row>
     <x:row r="164" ht="15" hidden="0" customHeight="1">
       <x:c r="A164" s="16" t="str">
-        <x:f>IF(AND(B164="",C164=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B164&amp;C164," ",""))&amp;IF(E164&lt;&gt;"","-"&amp;RIGHT(E164,4),IF(J164&lt;&gt;"","-"&amp;RIGHT(J164,4),"")))</x:f>
+        <x:f>IF(AND(B164="",C164=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B164&amp;C164," ",""))&amp;IF(E164&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E164," ",""),4),IF(J164&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J164," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B164" s="16"/>
       <x:c r="C164" s="16"/>
@@ -4757,7 +4757,7 @@
     </x:row>
     <x:row r="165" ht="15" hidden="0" customHeight="1">
       <x:c r="A165" s="16" t="str">
-        <x:f>IF(AND(B165="",C165=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B165&amp;C165," ",""))&amp;IF(E165&lt;&gt;"","-"&amp;RIGHT(E165,4),IF(J165&lt;&gt;"","-"&amp;RIGHT(J165,4),"")))</x:f>
+        <x:f>IF(AND(B165="",C165=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B165&amp;C165," ",""))&amp;IF(E165&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E165," ",""),4),IF(J165&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J165," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B165" s="16"/>
       <x:c r="C165" s="16"/>
@@ -4783,7 +4783,7 @@
     </x:row>
     <x:row r="166" ht="15" hidden="0" customHeight="1">
       <x:c r="A166" s="16" t="str">
-        <x:f>IF(AND(B166="",C166=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B166&amp;C166," ",""))&amp;IF(E166&lt;&gt;"","-"&amp;RIGHT(E166,4),IF(J166&lt;&gt;"","-"&amp;RIGHT(J166,4),"")))</x:f>
+        <x:f>IF(AND(B166="",C166=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B166&amp;C166," ",""))&amp;IF(E166&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E166," ",""),4),IF(J166&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J166," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B166" s="16"/>
       <x:c r="C166" s="16"/>
@@ -4809,7 +4809,7 @@
     </x:row>
     <x:row r="167" ht="15" hidden="0" customHeight="1">
       <x:c r="A167" s="16" t="str">
-        <x:f>IF(AND(B167="",C167=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B167&amp;C167," ",""))&amp;IF(E167&lt;&gt;"","-"&amp;RIGHT(E167,4),IF(J167&lt;&gt;"","-"&amp;RIGHT(J167,4),"")))</x:f>
+        <x:f>IF(AND(B167="",C167=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B167&amp;C167," ",""))&amp;IF(E167&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E167," ",""),4),IF(J167&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J167," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B167" s="16"/>
       <x:c r="C167" s="16"/>
@@ -4835,7 +4835,7 @@
     </x:row>
     <x:row r="168" ht="15" hidden="0" customHeight="1">
       <x:c r="A168" s="16" t="str">
-        <x:f>IF(AND(B168="",C168=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B168&amp;C168," ",""))&amp;IF(E168&lt;&gt;"","-"&amp;RIGHT(E168,4),IF(J168&lt;&gt;"","-"&amp;RIGHT(J168,4),"")))</x:f>
+        <x:f>IF(AND(B168="",C168=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B168&amp;C168," ",""))&amp;IF(E168&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E168," ",""),4),IF(J168&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J168," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B168" s="16"/>
       <x:c r="C168" s="16"/>
@@ -4861,7 +4861,7 @@
     </x:row>
     <x:row r="169" ht="15" hidden="0" customHeight="1">
       <x:c r="A169" s="16" t="str">
-        <x:f>IF(AND(B169="",C169=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B169&amp;C169," ",""))&amp;IF(E169&lt;&gt;"","-"&amp;RIGHT(E169,4),IF(J169&lt;&gt;"","-"&amp;RIGHT(J169,4),"")))</x:f>
+        <x:f>IF(AND(B169="",C169=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B169&amp;C169," ",""))&amp;IF(E169&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E169," ",""),4),IF(J169&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J169," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B169" s="16"/>
       <x:c r="C169" s="16"/>
@@ -4887,7 +4887,7 @@
     </x:row>
     <x:row r="170" ht="15" hidden="0" customHeight="1">
       <x:c r="A170" s="16" t="str">
-        <x:f>IF(AND(B170="",C170=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B170&amp;C170," ",""))&amp;IF(E170&lt;&gt;"","-"&amp;RIGHT(E170,4),IF(J170&lt;&gt;"","-"&amp;RIGHT(J170,4),"")))</x:f>
+        <x:f>IF(AND(B170="",C170=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B170&amp;C170," ",""))&amp;IF(E170&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E170," ",""),4),IF(J170&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J170," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B170" s="16"/>
       <x:c r="C170" s="16"/>
@@ -4913,7 +4913,7 @@
     </x:row>
     <x:row r="171" ht="15" hidden="0" customHeight="1">
       <x:c r="A171" s="16" t="str">
-        <x:f>IF(AND(B171="",C171=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B171&amp;C171," ",""))&amp;IF(E171&lt;&gt;"","-"&amp;RIGHT(E171,4),IF(J171&lt;&gt;"","-"&amp;RIGHT(J171,4),"")))</x:f>
+        <x:f>IF(AND(B171="",C171=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B171&amp;C171," ",""))&amp;IF(E171&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E171," ",""),4),IF(J171&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J171," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B171" s="16"/>
       <x:c r="C171" s="16"/>
@@ -4939,7 +4939,7 @@
     </x:row>
     <x:row r="172" ht="15" hidden="0" customHeight="1">
       <x:c r="A172" s="16" t="str">
-        <x:f>IF(AND(B172="",C172=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B172&amp;C172," ",""))&amp;IF(E172&lt;&gt;"","-"&amp;RIGHT(E172,4),IF(J172&lt;&gt;"","-"&amp;RIGHT(J172,4),"")))</x:f>
+        <x:f>IF(AND(B172="",C172=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B172&amp;C172," ",""))&amp;IF(E172&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E172," ",""),4),IF(J172&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J172," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B172" s="16"/>
       <x:c r="C172" s="16"/>
@@ -4965,7 +4965,7 @@
     </x:row>
     <x:row r="173" ht="15" hidden="0" customHeight="1">
       <x:c r="A173" s="16" t="str">
-        <x:f>IF(AND(B173="",C173=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B173&amp;C173," ",""))&amp;IF(E173&lt;&gt;"","-"&amp;RIGHT(E173,4),IF(J173&lt;&gt;"","-"&amp;RIGHT(J173,4),"")))</x:f>
+        <x:f>IF(AND(B173="",C173=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B173&amp;C173," ",""))&amp;IF(E173&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E173," ",""),4),IF(J173&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J173," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B173" s="16"/>
       <x:c r="C173" s="16"/>
@@ -4991,7 +4991,7 @@
     </x:row>
     <x:row r="174" ht="15" hidden="0" customHeight="1">
       <x:c r="A174" s="16" t="str">
-        <x:f>IF(AND(B174="",C174=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B174&amp;C174," ",""))&amp;IF(E174&lt;&gt;"","-"&amp;RIGHT(E174,4),IF(J174&lt;&gt;"","-"&amp;RIGHT(J174,4),"")))</x:f>
+        <x:f>IF(AND(B174="",C174=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B174&amp;C174," ",""))&amp;IF(E174&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E174," ",""),4),IF(J174&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J174," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B174" s="16"/>
       <x:c r="C174" s="16"/>
@@ -5017,7 +5017,7 @@
     </x:row>
     <x:row r="175" ht="15" hidden="0" customHeight="1">
       <x:c r="A175" s="16" t="str">
-        <x:f>IF(AND(B175="",C175=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B175&amp;C175," ",""))&amp;IF(E175&lt;&gt;"","-"&amp;RIGHT(E175,4),IF(J175&lt;&gt;"","-"&amp;RIGHT(J175,4),"")))</x:f>
+        <x:f>IF(AND(B175="",C175=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B175&amp;C175," ",""))&amp;IF(E175&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E175," ",""),4),IF(J175&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J175," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B175" s="16"/>
       <x:c r="C175" s="16"/>
@@ -5043,7 +5043,7 @@
     </x:row>
     <x:row r="176" ht="15" hidden="0" customHeight="1">
       <x:c r="A176" s="16" t="str">
-        <x:f>IF(AND(B176="",C176=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B176&amp;C176," ",""))&amp;IF(E176&lt;&gt;"","-"&amp;RIGHT(E176,4),IF(J176&lt;&gt;"","-"&amp;RIGHT(J176,4),"")))</x:f>
+        <x:f>IF(AND(B176="",C176=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B176&amp;C176," ",""))&amp;IF(E176&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E176," ",""),4),IF(J176&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J176," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B176" s="16"/>
       <x:c r="C176" s="16"/>
@@ -5069,7 +5069,7 @@
     </x:row>
     <x:row r="177" ht="15" hidden="0" customHeight="1">
       <x:c r="A177" s="16" t="str">
-        <x:f>IF(AND(B177="",C177=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B177&amp;C177," ",""))&amp;IF(E177&lt;&gt;"","-"&amp;RIGHT(E177,4),IF(J177&lt;&gt;"","-"&amp;RIGHT(J177,4),"")))</x:f>
+        <x:f>IF(AND(B177="",C177=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B177&amp;C177," ",""))&amp;IF(E177&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E177," ",""),4),IF(J177&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J177," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B177" s="16"/>
       <x:c r="C177" s="16"/>
@@ -5095,7 +5095,7 @@
     </x:row>
     <x:row r="178" ht="15" hidden="0" customHeight="1">
       <x:c r="A178" s="16" t="str">
-        <x:f>IF(AND(B178="",C178=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B178&amp;C178," ",""))&amp;IF(E178&lt;&gt;"","-"&amp;RIGHT(E178,4),IF(J178&lt;&gt;"","-"&amp;RIGHT(J178,4),"")))</x:f>
+        <x:f>IF(AND(B178="",C178=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B178&amp;C178," ",""))&amp;IF(E178&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E178," ",""),4),IF(J178&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J178," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B178" s="16"/>
       <x:c r="C178" s="16"/>
@@ -5121,7 +5121,7 @@
     </x:row>
     <x:row r="179" ht="15" hidden="0" customHeight="1">
       <x:c r="A179" s="16" t="str">
-        <x:f>IF(AND(B179="",C179=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B179&amp;C179," ",""))&amp;IF(E179&lt;&gt;"","-"&amp;RIGHT(E179,4),IF(J179&lt;&gt;"","-"&amp;RIGHT(J179,4),"")))</x:f>
+        <x:f>IF(AND(B179="",C179=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B179&amp;C179," ",""))&amp;IF(E179&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E179," ",""),4),IF(J179&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J179," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B179" s="16"/>
       <x:c r="C179" s="16"/>
@@ -5147,7 +5147,7 @@
     </x:row>
     <x:row r="180" ht="15" hidden="0" customHeight="1">
       <x:c r="A180" s="16" t="str">
-        <x:f>IF(AND(B180="",C180=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B180&amp;C180," ",""))&amp;IF(E180&lt;&gt;"","-"&amp;RIGHT(E180,4),IF(J180&lt;&gt;"","-"&amp;RIGHT(J180,4),"")))</x:f>
+        <x:f>IF(AND(B180="",C180=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B180&amp;C180," ",""))&amp;IF(E180&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E180," ",""),4),IF(J180&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J180," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B180" s="16"/>
       <x:c r="C180" s="16"/>
@@ -5173,7 +5173,7 @@
     </x:row>
     <x:row r="181" ht="15" hidden="0" customHeight="1">
       <x:c r="A181" s="16" t="str">
-        <x:f>IF(AND(B181="",C181=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B181&amp;C181," ",""))&amp;IF(E181&lt;&gt;"","-"&amp;RIGHT(E181,4),IF(J181&lt;&gt;"","-"&amp;RIGHT(J181,4),"")))</x:f>
+        <x:f>IF(AND(B181="",C181=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B181&amp;C181," ",""))&amp;IF(E181&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E181," ",""),4),IF(J181&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J181," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B181" s="16"/>
       <x:c r="C181" s="16"/>
@@ -5199,7 +5199,7 @@
     </x:row>
     <x:row r="182" ht="15" hidden="0" customHeight="1">
       <x:c r="A182" s="16" t="str">
-        <x:f>IF(AND(B182="",C182=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B182&amp;C182," ",""))&amp;IF(E182&lt;&gt;"","-"&amp;RIGHT(E182,4),IF(J182&lt;&gt;"","-"&amp;RIGHT(J182,4),"")))</x:f>
+        <x:f>IF(AND(B182="",C182=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B182&amp;C182," ",""))&amp;IF(E182&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E182," ",""),4),IF(J182&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J182," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B182" s="16"/>
       <x:c r="C182" s="16"/>
@@ -5225,7 +5225,7 @@
     </x:row>
     <x:row r="183" ht="15" hidden="0" customHeight="1">
       <x:c r="A183" s="16" t="str">
-        <x:f>IF(AND(B183="",C183=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B183&amp;C183," ",""))&amp;IF(E183&lt;&gt;"","-"&amp;RIGHT(E183,4),IF(J183&lt;&gt;"","-"&amp;RIGHT(J183,4),"")))</x:f>
+        <x:f>IF(AND(B183="",C183=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B183&amp;C183," ",""))&amp;IF(E183&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E183," ",""),4),IF(J183&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J183," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B183" s="16"/>
       <x:c r="C183" s="16"/>
@@ -5251,7 +5251,7 @@
     </x:row>
     <x:row r="184" ht="15" hidden="0" customHeight="1">
       <x:c r="A184" s="16" t="str">
-        <x:f>IF(AND(B184="",C184=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B184&amp;C184," ",""))&amp;IF(E184&lt;&gt;"","-"&amp;RIGHT(E184,4),IF(J184&lt;&gt;"","-"&amp;RIGHT(J184,4),"")))</x:f>
+        <x:f>IF(AND(B184="",C184=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B184&amp;C184," ",""))&amp;IF(E184&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E184," ",""),4),IF(J184&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J184," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B184" s="16"/>
       <x:c r="C184" s="16"/>
@@ -5277,7 +5277,7 @@
     </x:row>
     <x:row r="185" ht="15" hidden="0" customHeight="1">
       <x:c r="A185" s="16" t="str">
-        <x:f>IF(AND(B185="",C185=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B185&amp;C185," ",""))&amp;IF(E185&lt;&gt;"","-"&amp;RIGHT(E185,4),IF(J185&lt;&gt;"","-"&amp;RIGHT(J185,4),"")))</x:f>
+        <x:f>IF(AND(B185="",C185=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B185&amp;C185," ",""))&amp;IF(E185&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E185," ",""),4),IF(J185&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J185," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B185" s="16"/>
       <x:c r="C185" s="16"/>
@@ -5303,7 +5303,7 @@
     </x:row>
     <x:row r="186" ht="15" hidden="0" customHeight="1">
       <x:c r="A186" s="16" t="str">
-        <x:f>IF(AND(B186="",C186=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B186&amp;C186," ",""))&amp;IF(E186&lt;&gt;"","-"&amp;RIGHT(E186,4),IF(J186&lt;&gt;"","-"&amp;RIGHT(J186,4),"")))</x:f>
+        <x:f>IF(AND(B186="",C186=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B186&amp;C186," ",""))&amp;IF(E186&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E186," ",""),4),IF(J186&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J186," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B186" s="16"/>
       <x:c r="C186" s="16"/>
@@ -5329,7 +5329,7 @@
     </x:row>
     <x:row r="187" ht="15" hidden="0" customHeight="1">
       <x:c r="A187" s="16" t="str">
-        <x:f>IF(AND(B187="",C187=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B187&amp;C187," ",""))&amp;IF(E187&lt;&gt;"","-"&amp;RIGHT(E187,4),IF(J187&lt;&gt;"","-"&amp;RIGHT(J187,4),"")))</x:f>
+        <x:f>IF(AND(B187="",C187=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B187&amp;C187," ",""))&amp;IF(E187&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E187," ",""),4),IF(J187&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J187," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B187" s="16"/>
       <x:c r="C187" s="16"/>
@@ -5355,7 +5355,7 @@
     </x:row>
     <x:row r="188" ht="15" hidden="0" customHeight="1">
       <x:c r="A188" s="16" t="str">
-        <x:f>IF(AND(B188="",C188=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B188&amp;C188," ",""))&amp;IF(E188&lt;&gt;"","-"&amp;RIGHT(E188,4),IF(J188&lt;&gt;"","-"&amp;RIGHT(J188,4),"")))</x:f>
+        <x:f>IF(AND(B188="",C188=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B188&amp;C188," ",""))&amp;IF(E188&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E188," ",""),4),IF(J188&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J188," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B188" s="16"/>
       <x:c r="C188" s="16"/>
@@ -5381,7 +5381,7 @@
     </x:row>
     <x:row r="189" ht="15" hidden="0" customHeight="1">
       <x:c r="A189" s="16" t="str">
-        <x:f>IF(AND(B189="",C189=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B189&amp;C189," ",""))&amp;IF(E189&lt;&gt;"","-"&amp;RIGHT(E189,4),IF(J189&lt;&gt;"","-"&amp;RIGHT(J189,4),"")))</x:f>
+        <x:f>IF(AND(B189="",C189=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B189&amp;C189," ",""))&amp;IF(E189&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E189," ",""),4),IF(J189&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J189," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B189" s="16"/>
       <x:c r="C189" s="16"/>
@@ -5407,7 +5407,7 @@
     </x:row>
     <x:row r="190" ht="15" hidden="0" customHeight="1">
       <x:c r="A190" s="16" t="str">
-        <x:f>IF(AND(B190="",C190=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B190&amp;C190," ",""))&amp;IF(E190&lt;&gt;"","-"&amp;RIGHT(E190,4),IF(J190&lt;&gt;"","-"&amp;RIGHT(J190,4),"")))</x:f>
+        <x:f>IF(AND(B190="",C190=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B190&amp;C190," ",""))&amp;IF(E190&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E190," ",""),4),IF(J190&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J190," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B190" s="16"/>
       <x:c r="C190" s="16"/>
@@ -5433,7 +5433,7 @@
     </x:row>
     <x:row r="191" ht="15" hidden="0" customHeight="1">
       <x:c r="A191" s="16" t="str">
-        <x:f>IF(AND(B191="",C191=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B191&amp;C191," ",""))&amp;IF(E191&lt;&gt;"","-"&amp;RIGHT(E191,4),IF(J191&lt;&gt;"","-"&amp;RIGHT(J191,4),"")))</x:f>
+        <x:f>IF(AND(B191="",C191=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B191&amp;C191," ",""))&amp;IF(E191&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E191," ",""),4),IF(J191&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J191," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B191" s="16"/>
       <x:c r="C191" s="16"/>
@@ -5459,7 +5459,7 @@
     </x:row>
     <x:row r="192" ht="15" hidden="0" customHeight="1">
       <x:c r="A192" s="16" t="str">
-        <x:f>IF(AND(B192="",C192=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B192&amp;C192," ",""))&amp;IF(E192&lt;&gt;"","-"&amp;RIGHT(E192,4),IF(J192&lt;&gt;"","-"&amp;RIGHT(J192,4),"")))</x:f>
+        <x:f>IF(AND(B192="",C192=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B192&amp;C192," ",""))&amp;IF(E192&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E192," ",""),4),IF(J192&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J192," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B192" s="16"/>
       <x:c r="C192" s="16"/>
@@ -5485,7 +5485,7 @@
     </x:row>
     <x:row r="193" ht="15" hidden="0" customHeight="1">
       <x:c r="A193" s="16" t="str">
-        <x:f>IF(AND(B193="",C193=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B193&amp;C193," ",""))&amp;IF(E193&lt;&gt;"","-"&amp;RIGHT(E193,4),IF(J193&lt;&gt;"","-"&amp;RIGHT(J193,4),"")))</x:f>
+        <x:f>IF(AND(B193="",C193=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B193&amp;C193," ",""))&amp;IF(E193&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E193," ",""),4),IF(J193&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J193," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B193" s="16"/>
       <x:c r="C193" s="16"/>
@@ -5511,7 +5511,7 @@
     </x:row>
     <x:row r="194" ht="15" hidden="0" customHeight="1">
       <x:c r="A194" s="16" t="str">
-        <x:f>IF(AND(B194="",C194=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B194&amp;C194," ",""))&amp;IF(E194&lt;&gt;"","-"&amp;RIGHT(E194,4),IF(J194&lt;&gt;"","-"&amp;RIGHT(J194,4),"")))</x:f>
+        <x:f>IF(AND(B194="",C194=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B194&amp;C194," ",""))&amp;IF(E194&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E194," ",""),4),IF(J194&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J194," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B194" s="16"/>
       <x:c r="C194" s="16"/>
@@ -5537,7 +5537,7 @@
     </x:row>
     <x:row r="195" ht="15" hidden="0" customHeight="1">
       <x:c r="A195" s="16" t="str">
-        <x:f>IF(AND(B195="",C195=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B195&amp;C195," ",""))&amp;IF(E195&lt;&gt;"","-"&amp;RIGHT(E195,4),IF(J195&lt;&gt;"","-"&amp;RIGHT(J195,4),"")))</x:f>
+        <x:f>IF(AND(B195="",C195=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B195&amp;C195," ",""))&amp;IF(E195&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E195," ",""),4),IF(J195&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J195," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B195" s="16"/>
       <x:c r="C195" s="16"/>
@@ -5563,7 +5563,7 @@
     </x:row>
     <x:row r="196" ht="15" hidden="0" customHeight="1">
       <x:c r="A196" s="16" t="str">
-        <x:f>IF(AND(B196="",C196=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B196&amp;C196," ",""))&amp;IF(E196&lt;&gt;"","-"&amp;RIGHT(E196,4),IF(J196&lt;&gt;"","-"&amp;RIGHT(J196,4),"")))</x:f>
+        <x:f>IF(AND(B196="",C196=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B196&amp;C196," ",""))&amp;IF(E196&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E196," ",""),4),IF(J196&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J196," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B196" s="16"/>
       <x:c r="C196" s="16"/>
@@ -5589,7 +5589,7 @@
     </x:row>
     <x:row r="197" ht="15" hidden="0" customHeight="1">
       <x:c r="A197" s="16" t="str">
-        <x:f>IF(AND(B197="",C197=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B197&amp;C197," ",""))&amp;IF(E197&lt;&gt;"","-"&amp;RIGHT(E197,4),IF(J197&lt;&gt;"","-"&amp;RIGHT(J197,4),"")))</x:f>
+        <x:f>IF(AND(B197="",C197=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B197&amp;C197," ",""))&amp;IF(E197&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E197," ",""),4),IF(J197&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J197," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B197" s="16"/>
       <x:c r="C197" s="16"/>
@@ -5615,7 +5615,7 @@
     </x:row>
     <x:row r="198" ht="15" hidden="0" customHeight="1">
       <x:c r="A198" s="16" t="str">
-        <x:f>IF(AND(B198="",C198=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B198&amp;C198," ",""))&amp;IF(E198&lt;&gt;"","-"&amp;RIGHT(E198,4),IF(J198&lt;&gt;"","-"&amp;RIGHT(J198,4),"")))</x:f>
+        <x:f>IF(AND(B198="",C198=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B198&amp;C198," ",""))&amp;IF(E198&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E198," ",""),4),IF(J198&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J198," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B198" s="16"/>
       <x:c r="C198" s="16"/>
@@ -5641,7 +5641,7 @@
     </x:row>
     <x:row r="199" ht="15" hidden="0" customHeight="1">
       <x:c r="A199" s="16" t="str">
-        <x:f>IF(AND(B199="",C199=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B199&amp;C199," ",""))&amp;IF(E199&lt;&gt;"","-"&amp;RIGHT(E199,4),IF(J199&lt;&gt;"","-"&amp;RIGHT(J199,4),"")))</x:f>
+        <x:f>IF(AND(B199="",C199=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B199&amp;C199," ",""))&amp;IF(E199&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E199," ",""),4),IF(J199&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J199," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B199" s="16"/>
       <x:c r="C199" s="16"/>
@@ -5667,7 +5667,7 @@
     </x:row>
     <x:row r="200" ht="15" hidden="0" customHeight="1">
       <x:c r="A200" s="16" t="str">
-        <x:f>IF(AND(B200="",C200=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B200&amp;C200," ",""))&amp;IF(E200&lt;&gt;"","-"&amp;RIGHT(E200,4),IF(J200&lt;&gt;"","-"&amp;RIGHT(J200,4),"")))</x:f>
+        <x:f>IF(AND(B200="",C200=""),"","M"&amp;TEXT(ROW()-1,"000")&amp;"-"&amp;LOWER(SUBSTITUTE(B200&amp;C200," ",""))&amp;IF(E200&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(E200," ",""),4),IF(J200&lt;&gt;"","-"&amp;RIGHT(SUBSTITUTE(J200," ",""),4),"")))</x:f>
       </x:c>
       <x:c r="B200" s="16"/>
       <x:c r="C200" s="16"/>
@@ -5720,7 +5720,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f3f8906ae6b4f1c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd76e8612ac1948cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5755,7 +5755,7 @@
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A1" s="13" t="str">
-        <x:v>Référence auto (optionnel)</x:v>
+        <x:v>Code membre auto</x:v>
       </x:c>
       <x:c r="B1" s="13" t="str">
         <x:v>Prénom</x:v>
@@ -5889,7 +5889,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8dd1dd988084757"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf6a9afd07b2486b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6070,8 +6070,8 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red19380a6c1b4e76"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ca0e59a0d664a3e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0268c58894bd43ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbce4e07fb86d4d0e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6094,10 +6094,10 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="16" t="str">
-        <x:v>Référence auto</x:v>
+        <x:v>Code membre auto</x:v>
       </x:c>
       <x:c r="B2" s="16" t="str">
-        <x:v>Optionnelle. Laissez la formule, videz ou supprimez la colonne: l'application régénère une référence sûre à l'import.</x:v>
+        <x:v>Optionnel. Laissez la formule, videz ou supprimez la colonne: l'application régénère un code sûr à l'import.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -6183,7 +6183,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9aa5f0368fd4fe0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad29c6cbb133410e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6209,7 +6209,7 @@
         <x:v>externalId / reference / code / matricule</x:v>
       </x:c>
       <x:c r="B2" s="16" t="str">
-        <x:v>Référence auto (optionnel), ou aucune colonne</x:v>
+        <x:v>Code membre auto, ou aucune colonne</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -6303,7 +6303,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f12ece186aa47cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60a496bf01fc46ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>